<commit_message>
get data from excel
</commit_message>
<xml_diff>
--- a/src/excel_resources/excel_data.xlsx
+++ b/src/excel_resources/excel_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0096F69B-4092-4F6A-8C5A-42D95CF2F431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC5D553-17FE-4946-B674-2E2A9B8E2F58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="72">
   <si>
     <t>10A1</t>
   </si>
@@ -140,9 +140,6 @@
   </si>
   <si>
     <t>Tự Nhiên</t>
-  </si>
-  <si>
-    <t>Ban Giáo Hiệu</t>
   </si>
   <si>
     <t>Tên môn học</t>
@@ -282,7 +279,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -388,6 +385,15 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -407,13 +413,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -428,19 +436,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -748,8 +756,8 @@
   </cols>
   <sheetData>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="18" t="s">
-        <v>72</v>
+      <c r="A5" s="9" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -772,15 +780,15 @@
         <v>33</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="C7" s="1" t="str">
         <f>A47</f>
@@ -800,7 +808,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>12</v>
@@ -921,8 +929,8 @@
       <c r="G19" s="1"/>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A21" s="18" t="s">
-        <v>68</v>
+      <c r="A21" s="9" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.35">
@@ -934,26 +942,26 @@
       <c r="A23" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="13"/>
-      <c r="O23" s="13"/>
-      <c r="P23" s="13"/>
-      <c r="Q23" s="13"/>
-      <c r="R23" s="13"/>
-      <c r="S23" s="13"/>
-      <c r="T23" s="13"/>
-      <c r="U23" s="13"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="6"/>
+      <c r="S23" s="6"/>
+      <c r="T23" s="6"/>
+      <c r="U23" s="6"/>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
@@ -986,104 +994,104 @@
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34" s="17" t="s">
+      <c r="A34" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A36" s="17" t="s">
+      <c r="A36" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A37" s="17" t="s">
+      <c r="A37" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A38" s="17" t="s">
+      <c r="A38" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A39" s="17" t="s">
+      <c r="A39" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A41" s="17" t="s">
+      <c r="A41" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A42" s="17" t="s">
+      <c r="A42" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A44" s="19" t="s">
-        <v>69</v>
+      <c r="A44" s="10" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="C45" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="D45" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="E45" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="F45" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B46" s="2">
         <v>1</v>
       </c>
       <c r="C46" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" ref="C46:C62" si="0">A$81</f>
         <v>Sáng</v>
       </c>
       <c r="D46" s="2">
@@ -1100,13 +1108,13 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47" s="2">
         <v>1</v>
       </c>
       <c r="C47" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D47" s="2">
@@ -1123,13 +1131,13 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B48" s="2">
         <v>1</v>
       </c>
       <c r="C48" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D48" s="2">
@@ -1146,188 +1154,182 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B49" s="2">
         <v>1</v>
       </c>
       <c r="C49" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D49" s="2">
         <v>1</v>
       </c>
       <c r="E49" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" ref="E49:E62" si="1">B$82</f>
         <v>0</v>
       </c>
       <c r="F49" s="2" t="str">
         <f>A$66</f>
         <v>Xã Hội</v>
       </c>
-      <c r="G49" s="13"/>
+      <c r="G49" s="6"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B50" s="2">
         <v>1</v>
       </c>
       <c r="C50" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D50" s="2">
         <v>1</v>
       </c>
       <c r="E50" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F50" s="2" t="str">
         <f>A$66</f>
         <v>Xã Hội</v>
       </c>
-      <c r="G50" s="14"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B51" s="2">
         <v>1</v>
       </c>
       <c r="C51" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D51" s="2">
         <v>1</v>
       </c>
       <c r="E51" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F51" s="2" t="str">
         <f>A$67</f>
         <v>Tự Nhiên</v>
       </c>
-      <c r="G51" s="14"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B52" s="2">
         <v>1</v>
       </c>
       <c r="C52" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D52" s="2">
         <v>1</v>
       </c>
       <c r="E52" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F52" s="2" t="str">
         <f>A$67</f>
         <v>Tự Nhiên</v>
       </c>
-      <c r="G52" s="14"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B53" s="2">
         <v>1</v>
       </c>
       <c r="C53" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D53" s="2">
         <v>1</v>
       </c>
       <c r="E53" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F53" s="2" t="str">
         <f>A$67</f>
         <v>Tự Nhiên</v>
       </c>
-      <c r="G53" s="14"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B54" s="2">
         <v>2</v>
       </c>
       <c r="C54" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D54" s="2">
         <v>2</v>
       </c>
       <c r="E54" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F54" s="2" t="str">
         <f>A$67</f>
         <v>Tự Nhiên</v>
       </c>
-      <c r="G54" s="14"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B55" s="2">
         <v>2</v>
       </c>
       <c r="C55" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D55" s="2">
         <v>2</v>
       </c>
       <c r="E55" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F55" s="2" t="str">
         <f>A$66</f>
         <v>Xã Hội</v>
       </c>
-      <c r="G55" s="14"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B56" s="2">
         <v>1</v>
       </c>
       <c r="C56" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D56" s="2">
         <v>1</v>
       </c>
       <c r="E56" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F56" s="2" t="str">
@@ -1337,20 +1339,20 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B57" s="2">
         <v>2</v>
       </c>
       <c r="C57" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D57" s="2">
         <v>2</v>
       </c>
       <c r="E57" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F57" s="2" t="str">
@@ -1360,20 +1362,20 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B58" s="2">
         <v>2</v>
       </c>
       <c r="C58" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D58" s="2">
         <v>2</v>
       </c>
       <c r="E58" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F58" s="2" t="str">
@@ -1383,20 +1385,20 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B59" s="2">
         <v>2</v>
       </c>
       <c r="C59" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D59" s="2">
         <v>2</v>
       </c>
       <c r="E59" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F59" s="2" t="str">
@@ -1406,20 +1408,20 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B60" s="2">
         <v>2</v>
       </c>
       <c r="C60" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D60" s="2">
         <v>2</v>
       </c>
       <c r="E60" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F60" s="2" t="str">
@@ -1429,20 +1431,20 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B61" s="2">
         <v>1</v>
       </c>
       <c r="C61" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D61" s="2">
         <v>1</v>
       </c>
       <c r="E61" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F61" s="2" t="str">
@@ -1452,20 +1454,20 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B62" s="2">
         <v>1</v>
       </c>
       <c r="C62" s="2" t="str">
-        <f>A$81</f>
+        <f t="shared" si="0"/>
         <v>Sáng</v>
       </c>
       <c r="D62" s="2">
         <v>1</v>
       </c>
       <c r="E62" s="2" t="b">
-        <f>B$82</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F62" s="2" t="str">
@@ -1474,17 +1476,17 @@
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A64" s="18" t="s">
-        <v>70</v>
+      <c r="A64" s="9" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B65" s="15"/>
-      <c r="C65" s="13"/>
-      <c r="D65" s="13"/>
+      <c r="B65" s="7"/>
+      <c r="C65" s="6"/>
+      <c r="D65" s="6"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
@@ -1492,108 +1494,79 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A67" s="2" t="s">
+      <c r="A67" s="18" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A68" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C68" s="13"/>
-      <c r="D68" s="13"/>
-      <c r="E68" s="13"/>
-      <c r="F68" s="13"/>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C69" s="14"/>
-      <c r="D69" s="14"/>
-      <c r="E69" s="14"/>
-      <c r="F69" s="14"/>
+      <c r="A68" s="19"/>
+      <c r="C68" s="6"/>
+      <c r="D68" s="6"/>
+      <c r="E68" s="6"/>
+      <c r="F68" s="6"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A70" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="C70" s="14"/>
-      <c r="D70" s="14"/>
-      <c r="E70" s="14"/>
-      <c r="F70" s="14"/>
+      <c r="A70" s="10" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="B71" s="15"/>
-      <c r="C71" s="14"/>
-      <c r="D71" s="14"/>
-      <c r="E71" s="14"/>
-      <c r="F71" s="14"/>
+        <v>64</v>
+      </c>
+      <c r="B71" s="7"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B72" s="16"/>
-      <c r="C72" s="14"/>
-      <c r="D72" s="14"/>
-      <c r="E72" s="14"/>
-      <c r="F72" s="14"/>
+      <c r="B72" s="8"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B73" s="16"/>
-      <c r="C73" s="14"/>
-      <c r="D73" s="14"/>
-      <c r="E73" s="14"/>
-      <c r="F73" s="14"/>
+      <c r="B73" s="8"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B74" s="16"/>
-      <c r="C74" s="14"/>
-      <c r="D74" s="14"/>
-      <c r="E74" s="14"/>
-      <c r="F74" s="14"/>
+      <c r="B74" s="8"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B75" s="16"/>
+      <c r="B75" s="8"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B76" s="16"/>
+      <c r="B76" s="8"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B77" s="16"/>
-      <c r="C77" s="13"/>
+      <c r="B77" s="8"/>
+      <c r="C77" s="6"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C78" s="13"/>
+      <c r="C78" s="6"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A79" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="C79" s="14"/>
+      <c r="A79" s="9" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B80" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.35">
@@ -1606,7 +1579,7 @@
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A82" s="17" t="s">
+      <c r="A82" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B82" s="1" t="b">
@@ -1626,28 +1599,28 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7"/>
-      <c r="R4" s="7"/>
-      <c r="S4" s="7"/>
-      <c r="T4" s="7"/>
-      <c r="U4" s="7"/>
-      <c r="V4" s="8"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="16"/>
+      <c r="N4" s="16"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="16"/>
+      <c r="Q4" s="16"/>
+      <c r="R4" s="16"/>
+      <c r="S4" s="16"/>
+      <c r="T4" s="16"/>
+      <c r="U4" s="16"/>
+      <c r="V4" s="17"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
@@ -1713,7 +1686,7 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="3">
@@ -1741,7 +1714,7 @@
       <c r="V6" s="1"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A7" s="9"/>
+      <c r="A7" s="11"/>
       <c r="B7" s="3">
         <v>2</v>
       </c>
@@ -1767,7 +1740,7 @@
       <c r="V7" s="1"/>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A8" s="9"/>
+      <c r="A8" s="11"/>
       <c r="B8" s="3">
         <v>3</v>
       </c>
@@ -1793,7 +1766,7 @@
       <c r="V8" s="1"/>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A9" s="9"/>
+      <c r="A9" s="11"/>
       <c r="B9" s="3">
         <v>4</v>
       </c>
@@ -1819,7 +1792,7 @@
       <c r="V9" s="1"/>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A10" s="9"/>
+      <c r="A10" s="11"/>
       <c r="B10" s="3">
         <v>5</v>
       </c>
@@ -1845,7 +1818,7 @@
       <c r="V10" s="1"/>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="3">
@@ -1873,7 +1846,7 @@
       <c r="V11" s="1"/>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="11"/>
+      <c r="A12" s="13"/>
       <c r="B12" s="4">
         <v>7</v>
       </c>
@@ -1899,7 +1872,7 @@
       <c r="V12" s="1"/>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A13" s="12"/>
+      <c r="A13" s="14"/>
       <c r="B13" s="4">
         <v>8</v>
       </c>
@@ -1925,28 +1898,28 @@
       <c r="V13" s="1"/>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="7"/>
-      <c r="N16" s="7"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="7"/>
-      <c r="Q16" s="7"/>
-      <c r="R16" s="7"/>
-      <c r="S16" s="7"/>
-      <c r="T16" s="7"/>
-      <c r="U16" s="7"/>
-      <c r="V16" s="8"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="16"/>
+      <c r="P16" s="16"/>
+      <c r="Q16" s="16"/>
+      <c r="R16" s="16"/>
+      <c r="S16" s="16"/>
+      <c r="T16" s="16"/>
+      <c r="U16" s="16"/>
+      <c r="V16" s="17"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -2012,7 +1985,7 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="3">
@@ -2040,7 +2013,7 @@
       <c r="V18" s="1"/>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A19" s="9"/>
+      <c r="A19" s="11"/>
       <c r="B19" s="3">
         <v>2</v>
       </c>
@@ -2066,7 +2039,7 @@
       <c r="V19" s="1"/>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A20" s="9"/>
+      <c r="A20" s="11"/>
       <c r="B20" s="3">
         <v>3</v>
       </c>
@@ -2092,7 +2065,7 @@
       <c r="V20" s="1"/>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A21" s="9"/>
+      <c r="A21" s="11"/>
       <c r="B21" s="3">
         <v>4</v>
       </c>
@@ -2118,7 +2091,7 @@
       <c r="V21" s="1"/>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A22" s="9"/>
+      <c r="A22" s="11"/>
       <c r="B22" s="3">
         <v>5</v>
       </c>
@@ -2144,7 +2117,7 @@
       <c r="V22" s="1"/>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="3">
@@ -2172,7 +2145,7 @@
       <c r="V23" s="1"/>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A24" s="11"/>
+      <c r="A24" s="13"/>
       <c r="B24" s="4">
         <v>7</v>
       </c>
@@ -2198,7 +2171,7 @@
       <c r="V24" s="1"/>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A25" s="12"/>
+      <c r="A25" s="14"/>
       <c r="B25" s="4">
         <v>8</v>
       </c>
@@ -2224,28 +2197,28 @@
       <c r="V25" s="1"/>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7"/>
-      <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
-      <c r="L28" s="7"/>
-      <c r="M28" s="7"/>
-      <c r="N28" s="7"/>
-      <c r="O28" s="7"/>
-      <c r="P28" s="7"/>
-      <c r="Q28" s="7"/>
-      <c r="R28" s="7"/>
-      <c r="S28" s="7"/>
-      <c r="T28" s="7"/>
-      <c r="U28" s="7"/>
-      <c r="V28" s="8"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="16"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="16"/>
+      <c r="M28" s="16"/>
+      <c r="N28" s="16"/>
+      <c r="O28" s="16"/>
+      <c r="P28" s="16"/>
+      <c r="Q28" s="16"/>
+      <c r="R28" s="16"/>
+      <c r="S28" s="16"/>
+      <c r="T28" s="16"/>
+      <c r="U28" s="16"/>
+      <c r="V28" s="17"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B29" s="1"/>
@@ -2311,7 +2284,7 @@
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="9" t="s">
+      <c r="A30" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="3">
@@ -2339,7 +2312,7 @@
       <c r="V30" s="1"/>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A31" s="9"/>
+      <c r="A31" s="11"/>
       <c r="B31" s="3">
         <v>2</v>
       </c>
@@ -2365,7 +2338,7 @@
       <c r="V31" s="1"/>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A32" s="9"/>
+      <c r="A32" s="11"/>
       <c r="B32" s="3">
         <v>3</v>
       </c>
@@ -2391,7 +2364,7 @@
       <c r="V32" s="1"/>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="9"/>
+      <c r="A33" s="11"/>
       <c r="B33" s="3">
         <v>4</v>
       </c>
@@ -2417,7 +2390,7 @@
       <c r="V33" s="1"/>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" s="9"/>
+      <c r="A34" s="11"/>
       <c r="B34" s="3">
         <v>5</v>
       </c>
@@ -2443,7 +2416,7 @@
       <c r="V34" s="1"/>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="3">
@@ -2471,7 +2444,7 @@
       <c r="V35" s="1"/>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="11"/>
+      <c r="A36" s="13"/>
       <c r="B36" s="4">
         <v>7</v>
       </c>
@@ -2497,7 +2470,7 @@
       <c r="V36" s="1"/>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="12"/>
+      <c r="A37" s="14"/>
       <c r="B37" s="4">
         <v>8</v>
       </c>
@@ -2523,28 +2496,28 @@
       <c r="V37" s="1"/>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="7"/>
-      <c r="E40" s="7"/>
-      <c r="F40" s="7"/>
-      <c r="G40" s="7"/>
-      <c r="H40" s="7"/>
-      <c r="I40" s="7"/>
-      <c r="J40" s="7"/>
-      <c r="K40" s="7"/>
-      <c r="L40" s="7"/>
-      <c r="M40" s="7"/>
-      <c r="N40" s="7"/>
-      <c r="O40" s="7"/>
-      <c r="P40" s="7"/>
-      <c r="Q40" s="7"/>
-      <c r="R40" s="7"/>
-      <c r="S40" s="7"/>
-      <c r="T40" s="7"/>
-      <c r="U40" s="7"/>
-      <c r="V40" s="8"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
+      <c r="I40" s="16"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="16"/>
+      <c r="L40" s="16"/>
+      <c r="M40" s="16"/>
+      <c r="N40" s="16"/>
+      <c r="O40" s="16"/>
+      <c r="P40" s="16"/>
+      <c r="Q40" s="16"/>
+      <c r="R40" s="16"/>
+      <c r="S40" s="16"/>
+      <c r="T40" s="16"/>
+      <c r="U40" s="16"/>
+      <c r="V40" s="17"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B41" s="1"/>
@@ -2610,7 +2583,7 @@
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="9" t="s">
+      <c r="A42" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="3">
@@ -2638,7 +2611,7 @@
       <c r="V42" s="1"/>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="9"/>
+      <c r="A43" s="11"/>
       <c r="B43" s="3">
         <v>2</v>
       </c>
@@ -2664,7 +2637,7 @@
       <c r="V43" s="1"/>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="9"/>
+      <c r="A44" s="11"/>
       <c r="B44" s="3">
         <v>3</v>
       </c>
@@ -2690,7 +2663,7 @@
       <c r="V44" s="1"/>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" s="9"/>
+      <c r="A45" s="11"/>
       <c r="B45" s="3">
         <v>4</v>
       </c>
@@ -2716,7 +2689,7 @@
       <c r="V45" s="1"/>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A46" s="9"/>
+      <c r="A46" s="11"/>
       <c r="B46" s="3">
         <v>5</v>
       </c>
@@ -2742,7 +2715,7 @@
       <c r="V46" s="1"/>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="10" t="s">
+      <c r="A47" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B47" s="3">
@@ -2770,7 +2743,7 @@
       <c r="V47" s="1"/>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="11"/>
+      <c r="A48" s="13"/>
       <c r="B48" s="4">
         <v>7</v>
       </c>
@@ -2796,7 +2769,7 @@
       <c r="V48" s="1"/>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A49" s="12"/>
+      <c r="A49" s="14"/>
       <c r="B49" s="4">
         <v>8</v>
       </c>
@@ -2822,28 +2795,28 @@
       <c r="V49" s="1"/>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="7"/>
-      <c r="E52" s="7"/>
-      <c r="F52" s="7"/>
-      <c r="G52" s="7"/>
-      <c r="H52" s="7"/>
-      <c r="I52" s="7"/>
-      <c r="J52" s="7"/>
-      <c r="K52" s="7"/>
-      <c r="L52" s="7"/>
-      <c r="M52" s="7"/>
-      <c r="N52" s="7"/>
-      <c r="O52" s="7"/>
-      <c r="P52" s="7"/>
-      <c r="Q52" s="7"/>
-      <c r="R52" s="7"/>
-      <c r="S52" s="7"/>
-      <c r="T52" s="7"/>
-      <c r="U52" s="7"/>
-      <c r="V52" s="8"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
+      <c r="F52" s="16"/>
+      <c r="G52" s="16"/>
+      <c r="H52" s="16"/>
+      <c r="I52" s="16"/>
+      <c r="J52" s="16"/>
+      <c r="K52" s="16"/>
+      <c r="L52" s="16"/>
+      <c r="M52" s="16"/>
+      <c r="N52" s="16"/>
+      <c r="O52" s="16"/>
+      <c r="P52" s="16"/>
+      <c r="Q52" s="16"/>
+      <c r="R52" s="16"/>
+      <c r="S52" s="16"/>
+      <c r="T52" s="16"/>
+      <c r="U52" s="16"/>
+      <c r="V52" s="17"/>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B53" s="1"/>
@@ -2909,7 +2882,7 @@
       </c>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A54" s="9" t="s">
+      <c r="A54" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="3">
@@ -2937,7 +2910,7 @@
       <c r="V54" s="1"/>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A55" s="9"/>
+      <c r="A55" s="11"/>
       <c r="B55" s="3">
         <v>2</v>
       </c>
@@ -2963,7 +2936,7 @@
       <c r="V55" s="1"/>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A56" s="9"/>
+      <c r="A56" s="11"/>
       <c r="B56" s="3">
         <v>3</v>
       </c>
@@ -2989,7 +2962,7 @@
       <c r="V56" s="1"/>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" s="9"/>
+      <c r="A57" s="11"/>
       <c r="B57" s="3">
         <v>4</v>
       </c>
@@ -3015,7 +2988,7 @@
       <c r="V57" s="1"/>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A58" s="9"/>
+      <c r="A58" s="11"/>
       <c r="B58" s="3">
         <v>5</v>
       </c>
@@ -3041,7 +3014,7 @@
       <c r="V58" s="1"/>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="10" t="s">
+      <c r="A59" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B59" s="3">
@@ -3069,7 +3042,7 @@
       <c r="V59" s="1"/>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="11"/>
+      <c r="A60" s="13"/>
       <c r="B60" s="4">
         <v>7</v>
       </c>
@@ -3095,7 +3068,7 @@
       <c r="V60" s="1"/>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="12"/>
+      <c r="A61" s="14"/>
       <c r="B61" s="4">
         <v>8</v>
       </c>
@@ -3121,28 +3094,28 @@
       <c r="V61" s="1"/>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C64" s="6" t="s">
+      <c r="C64" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="D64" s="7"/>
-      <c r="E64" s="7"/>
-      <c r="F64" s="7"/>
-      <c r="G64" s="7"/>
-      <c r="H64" s="7"/>
-      <c r="I64" s="7"/>
-      <c r="J64" s="7"/>
-      <c r="K64" s="7"/>
-      <c r="L64" s="7"/>
-      <c r="M64" s="7"/>
-      <c r="N64" s="7"/>
-      <c r="O64" s="7"/>
-      <c r="P64" s="7"/>
-      <c r="Q64" s="7"/>
-      <c r="R64" s="7"/>
-      <c r="S64" s="7"/>
-      <c r="T64" s="7"/>
-      <c r="U64" s="7"/>
-      <c r="V64" s="8"/>
+      <c r="D64" s="16"/>
+      <c r="E64" s="16"/>
+      <c r="F64" s="16"/>
+      <c r="G64" s="16"/>
+      <c r="H64" s="16"/>
+      <c r="I64" s="16"/>
+      <c r="J64" s="16"/>
+      <c r="K64" s="16"/>
+      <c r="L64" s="16"/>
+      <c r="M64" s="16"/>
+      <c r="N64" s="16"/>
+      <c r="O64" s="16"/>
+      <c r="P64" s="16"/>
+      <c r="Q64" s="16"/>
+      <c r="R64" s="16"/>
+      <c r="S64" s="16"/>
+      <c r="T64" s="16"/>
+      <c r="U64" s="16"/>
+      <c r="V64" s="17"/>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B65" s="1"/>
@@ -3208,7 +3181,7 @@
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="9" t="s">
+      <c r="A66" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B66" s="3">
@@ -3236,7 +3209,7 @@
       <c r="V66" s="1"/>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="9"/>
+      <c r="A67" s="11"/>
       <c r="B67" s="3">
         <v>2</v>
       </c>
@@ -3262,7 +3235,7 @@
       <c r="V67" s="1"/>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" s="9"/>
+      <c r="A68" s="11"/>
       <c r="B68" s="3">
         <v>3</v>
       </c>
@@ -3288,7 +3261,7 @@
       <c r="V68" s="1"/>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="9"/>
+      <c r="A69" s="11"/>
       <c r="B69" s="3">
         <v>4</v>
       </c>
@@ -3314,7 +3287,7 @@
       <c r="V69" s="1"/>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="9"/>
+      <c r="A70" s="11"/>
       <c r="B70" s="3">
         <v>5</v>
       </c>
@@ -3340,7 +3313,7 @@
       <c r="V70" s="1"/>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A71" s="10" t="s">
+      <c r="A71" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B71" s="3">
@@ -3368,7 +3341,7 @@
       <c r="V71" s="1"/>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="11"/>
+      <c r="A72" s="13"/>
       <c r="B72" s="4">
         <v>7</v>
       </c>
@@ -3394,7 +3367,7 @@
       <c r="V72" s="1"/>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" s="12"/>
+      <c r="A73" s="14"/>
       <c r="B73" s="4">
         <v>8</v>
       </c>
@@ -3421,6 +3394,16 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C4:V4"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="C16:V16"/>
+    <mergeCell ref="A18:A22"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C28:V28"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="C64:V64"/>
     <mergeCell ref="A66:A70"/>
     <mergeCell ref="A71:A73"/>
     <mergeCell ref="C40:V40"/>
@@ -3429,16 +3412,6 @@
     <mergeCell ref="C52:V52"/>
     <mergeCell ref="A54:A58"/>
     <mergeCell ref="A59:A61"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C28:V28"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="C64:V64"/>
-    <mergeCell ref="C4:V4"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="C16:V16"/>
-    <mergeCell ref="A18:A22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
first avoid unexpected lesson
</commit_message>
<xml_diff>
--- a/src/excel_resources/excel_data.xlsx
+++ b/src/excel_resources/excel_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91747D2B-3DBC-4F0C-A233-649DBC7E0427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92742E33-99B4-423C-8B85-0F1B3B7551B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4800" yWindow="0" windowWidth="14400" windowHeight="7810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="input" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4081" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2163" uniqueCount="101">
   <si>
     <t>10A1</t>
   </si>
@@ -251,9 +251,6 @@
   </si>
   <si>
     <t>Mã Đức Bảo-Văn</t>
-  </si>
-  <si>
-    <t>Mã Đức Bảo-CD Văn</t>
   </si>
   <si>
     <t>Hoàng Hiếu Trình</t>
@@ -534,6 +531,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -545,15 +551,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -908,7 +905,7 @@
         <v>105</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G7" s="13" t="str">
         <f>A117</f>
@@ -937,7 +934,7 @@
         <v>35</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G8" s="13" t="str">
         <f t="shared" ref="G8:G18" si="1">A$117</f>
@@ -950,10 +947,10 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C9" s="13" t="str">
         <f>A$89</f>
@@ -966,7 +963,7 @@
         <v>105</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G9" s="13" t="str">
         <f t="shared" si="1"/>
@@ -979,7 +976,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>6</v>
@@ -994,7 +991,7 @@
         <v>35</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G10" s="13" t="str">
         <f t="shared" si="1"/>
@@ -1007,10 +1004,10 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C11" s="13" t="str">
         <f>A$89</f>
@@ -1022,7 +1019,9 @@
       <c r="E11" s="13">
         <v>105</v>
       </c>
-      <c r="F11" s="13"/>
+      <c r="F11" s="13" t="s">
+        <v>99</v>
+      </c>
       <c r="G11" s="13" t="str">
         <f t="shared" si="1"/>
         <v>Thứ Năm</v>
@@ -1034,10 +1033,10 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="13" t="s">
         <v>77</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>78</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>55</v>
@@ -1048,7 +1047,9 @@
       <c r="E12" s="13">
         <v>35</v>
       </c>
-      <c r="F12" s="13"/>
+      <c r="F12" s="13" t="s">
+        <v>99</v>
+      </c>
       <c r="G12" s="13" t="str">
         <f t="shared" si="1"/>
         <v>Thứ Năm</v>
@@ -1060,10 +1061,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="13" t="s">
         <v>79</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>80</v>
       </c>
       <c r="C13" s="13" t="str">
         <f>A$89</f>
@@ -1087,10 +1088,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C14" s="13" t="s">
         <v>55</v>
@@ -1113,10 +1114,10 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C15" s="13" t="str">
         <f>A$91</f>
@@ -1140,10 +1141,10 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="13" t="s">
         <v>84</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>85</v>
       </c>
       <c r="C16" s="13" t="str">
         <f>A$100</f>
@@ -1167,10 +1168,10 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="C17" s="13" t="str">
         <f>A$91</f>
@@ -1194,10 +1195,10 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C18" s="13" t="str">
         <f>A$100</f>
@@ -2018,28 +2019,28 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="23"/>
-      <c r="R4" s="23"/>
-      <c r="S4" s="23"/>
-      <c r="T4" s="23"/>
-      <c r="U4" s="23"/>
-      <c r="V4" s="24"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="20"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
@@ -2105,41 +2106,41 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="3">
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>91</v>
-      </c>
       <c r="F6" s="1" t="s">
         <v>73</v>
       </c>
       <c r="G6" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="L6" s="1" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="M6" s="1" t="s">
         <v>73</v>
@@ -2173,42 +2174,42 @@
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A7" s="18"/>
+      <c r="A7" s="21"/>
       <c r="B7" s="3">
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="H7" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I7" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="L7" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="M7" s="1" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>73</v>
@@ -2239,45 +2240,45 @@
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A8" s="18"/>
+      <c r="A8" s="21"/>
       <c r="B8" s="3">
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="I8" s="1" t="s">
         <v>73</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L8" s="1" t="s">
         <v>73</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>73</v>
@@ -2286,17 +2287,17 @@
         <v>73</v>
       </c>
       <c r="Q8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="T8" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="R8" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="S8" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="U8" s="1" t="s">
         <v>73</v>
       </c>
@@ -2305,63 +2306,63 @@
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A9" s="18"/>
+      <c r="A9" s="21"/>
       <c r="B9" s="3">
         <v>4</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q9" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="O9" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q9" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="R9" s="1" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="S9" s="1" t="s">
         <v>73</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="U9" s="1" t="s">
         <v>73</v>
@@ -2371,7 +2372,7 @@
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A10" s="18"/>
+      <c r="A10" s="21"/>
       <c r="B10" s="3">
         <v>5</v>
       </c>
@@ -2379,7 +2380,7 @@
         <v>73</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>73</v>
@@ -2388,56 +2389,56 @@
         <v>73</v>
       </c>
       <c r="G10" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q10" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R10" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="N10" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="O10" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="P10" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q10" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="R10" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="S10" s="1" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="T10" s="1" t="s">
         <v>73</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="3">
@@ -2505,7 +2506,7 @@
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="20"/>
+      <c r="A12" s="23"/>
       <c r="B12" s="4">
         <v>7</v>
       </c>
@@ -2571,7 +2572,7 @@
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A13" s="21"/>
+      <c r="A13" s="24"/>
       <c r="B13" s="4">
         <v>8</v>
       </c>
@@ -2637,28 +2638,28 @@
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="23"/>
-      <c r="Q16" s="23"/>
-      <c r="R16" s="23"/>
-      <c r="S16" s="23"/>
-      <c r="T16" s="23"/>
-      <c r="U16" s="23"/>
-      <c r="V16" s="24"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
+      <c r="O16" s="19"/>
+      <c r="P16" s="19"/>
+      <c r="Q16" s="19"/>
+      <c r="R16" s="19"/>
+      <c r="S16" s="19"/>
+      <c r="T16" s="19"/>
+      <c r="U16" s="19"/>
+      <c r="V16" s="20"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -2724,41 +2725,41 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="3">
         <v>1</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>91</v>
-      </c>
       <c r="F18" s="1" t="s">
         <v>73</v>
       </c>
       <c r="G18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I18" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H18" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K18" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="J18" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="K18" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="L18" s="1" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="M18" s="1" t="s">
         <v>73</v>
@@ -2792,42 +2793,42 @@
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A19" s="18"/>
+      <c r="A19" s="21"/>
       <c r="B19" s="3">
         <v>2</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G19" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="H19" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I19" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="J19" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="L19" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="J19" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="M19" s="1" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="N19" s="1" t="s">
         <v>73</v>
@@ -2858,45 +2859,45 @@
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A20" s="18"/>
+      <c r="A20" s="21"/>
       <c r="B20" s="3">
         <v>3</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E20" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F20" s="1" t="s">
+      <c r="G20" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H20" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="G20" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="I20" s="1" t="s">
         <v>73</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L20" s="1" t="s">
         <v>73</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="O20" s="1" t="s">
         <v>73</v>
@@ -2905,17 +2906,17 @@
         <v>73</v>
       </c>
       <c r="Q20" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R20" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="S20" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="T20" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="R20" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="S20" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="T20" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="U20" s="1" t="s">
         <v>73</v>
       </c>
@@ -2924,63 +2925,63 @@
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A21" s="18"/>
+      <c r="A21" s="21"/>
       <c r="B21" s="3">
         <v>4</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="P21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q21" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="G21" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="L21" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="M21" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="N21" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="O21" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="P21" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q21" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="R21" s="1" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="S21" s="1" t="s">
         <v>73</v>
       </c>
       <c r="T21" s="1" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="U21" s="1" t="s">
         <v>73</v>
@@ -2990,7 +2991,7 @@
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A22" s="18"/>
+      <c r="A22" s="21"/>
       <c r="B22" s="3">
         <v>5</v>
       </c>
@@ -2998,7 +2999,7 @@
         <v>73</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>73</v>
@@ -3007,56 +3008,56 @@
         <v>73</v>
       </c>
       <c r="G22" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="P22" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q22" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R22" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="H22" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K22" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="L22" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="M22" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="N22" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="O22" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="P22" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q22" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="R22" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="S22" s="1" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="T22" s="1" t="s">
         <v>73</v>
       </c>
       <c r="U22" s="1" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="V22" s="1" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="3">
@@ -3124,7 +3125,7 @@
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A24" s="20"/>
+      <c r="A24" s="23"/>
       <c r="B24" s="4">
         <v>7</v>
       </c>
@@ -3190,7 +3191,7 @@
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A25" s="21"/>
+      <c r="A25" s="24"/>
       <c r="B25" s="4">
         <v>8</v>
       </c>
@@ -3256,28 +3257,28 @@
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="23"/>
-      <c r="K28" s="23"/>
-      <c r="L28" s="23"/>
-      <c r="M28" s="23"/>
-      <c r="N28" s="23"/>
-      <c r="O28" s="23"/>
-      <c r="P28" s="23"/>
-      <c r="Q28" s="23"/>
-      <c r="R28" s="23"/>
-      <c r="S28" s="23"/>
-      <c r="T28" s="23"/>
-      <c r="U28" s="23"/>
-      <c r="V28" s="24"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="19"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="19"/>
+      <c r="N28" s="19"/>
+      <c r="O28" s="19"/>
+      <c r="P28" s="19"/>
+      <c r="Q28" s="19"/>
+      <c r="R28" s="19"/>
+      <c r="S28" s="19"/>
+      <c r="T28" s="19"/>
+      <c r="U28" s="19"/>
+      <c r="V28" s="20"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B29" s="1"/>
@@ -3343,75 +3344,75 @@
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="3">
         <v>1</v>
       </c>
       <c r="C30" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="M30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="P30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="S30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="T30" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="K30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="L30" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="M30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="N30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="O30" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="P30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="R30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="S30" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="T30" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="U30" s="1" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="V30" s="1" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A31" s="18"/>
+      <c r="A31" s="21"/>
       <c r="B31" s="3">
         <v>2</v>
       </c>
@@ -3419,55 +3420,55 @@
         <v>73</v>
       </c>
       <c r="D31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="P31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="S31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="T31" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K31" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="L31" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="N31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="O31" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="P31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="R31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="S31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="T31" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="U31" s="1" t="s">
         <v>93</v>
@@ -3477,7 +3478,7 @@
       </c>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A32" s="18"/>
+      <c r="A32" s="21"/>
       <c r="B32" s="3">
         <v>3</v>
       </c>
@@ -3485,65 +3486,65 @@
         <v>73</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="E32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="P32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="S32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="T32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="U32" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="I32" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J32" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K32" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="L32" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="M32" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="N32" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="O32" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="P32" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q32" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="R32" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="S32" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="T32" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="U32" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="V32" s="1" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="18"/>
+      <c r="A33" s="21"/>
       <c r="B33" s="3">
         <v>4</v>
       </c>
@@ -3551,37 +3552,37 @@
         <v>73</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="G33" s="1" t="s">
         <v>73</v>
       </c>
       <c r="H33" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I33" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="I33" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="J33" s="1" t="s">
         <v>73</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
       <c r="O33" s="1" t="s">
         <v>73</v>
@@ -3590,7 +3591,7 @@
         <v>73</v>
       </c>
       <c r="Q33" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="R33" s="1" t="s">
         <v>73</v>
@@ -3605,11 +3606,11 @@
         <v>73</v>
       </c>
       <c r="V33" s="1" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" s="18"/>
+      <c r="A34" s="21"/>
       <c r="B34" s="3">
         <v>5</v>
       </c>
@@ -3623,7 +3624,7 @@
         <v>73</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>73</v>
@@ -3632,7 +3633,7 @@
         <v>73</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>73</v>
@@ -3641,16 +3642,16 @@
         <v>73</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="P34" s="1" t="s">
         <v>73</v>
@@ -3659,10 +3660,10 @@
         <v>73</v>
       </c>
       <c r="R34" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="S34" s="1" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="T34" s="1" t="s">
         <v>73</v>
@@ -3675,7 +3676,7 @@
       </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="3">
@@ -3743,7 +3744,7 @@
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="20"/>
+      <c r="A36" s="23"/>
       <c r="B36" s="4">
         <v>7</v>
       </c>
@@ -3809,7 +3810,7 @@
       </c>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="21"/>
+      <c r="A37" s="24"/>
       <c r="B37" s="4">
         <v>8</v>
       </c>
@@ -3875,28 +3876,28 @@
       </c>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C40" s="22" t="s">
+      <c r="C40" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="23"/>
-      <c r="E40" s="23"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
-      <c r="H40" s="23"/>
-      <c r="I40" s="23"/>
-      <c r="J40" s="23"/>
-      <c r="K40" s="23"/>
-      <c r="L40" s="23"/>
-      <c r="M40" s="23"/>
-      <c r="N40" s="23"/>
-      <c r="O40" s="23"/>
-      <c r="P40" s="23"/>
-      <c r="Q40" s="23"/>
-      <c r="R40" s="23"/>
-      <c r="S40" s="23"/>
-      <c r="T40" s="23"/>
-      <c r="U40" s="23"/>
-      <c r="V40" s="24"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="19"/>
+      <c r="H40" s="19"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="19"/>
+      <c r="K40" s="19"/>
+      <c r="L40" s="19"/>
+      <c r="M40" s="19"/>
+      <c r="N40" s="19"/>
+      <c r="O40" s="19"/>
+      <c r="P40" s="19"/>
+      <c r="Q40" s="19"/>
+      <c r="R40" s="19"/>
+      <c r="S40" s="19"/>
+      <c r="T40" s="19"/>
+      <c r="U40" s="19"/>
+      <c r="V40" s="20"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B41" s="1"/>
@@ -3962,7 +3963,7 @@
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="18" t="s">
+      <c r="A42" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="3">
@@ -4030,7 +4031,7 @@
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="18"/>
+      <c r="A43" s="21"/>
       <c r="B43" s="3">
         <v>2</v>
       </c>
@@ -4096,7 +4097,7 @@
       </c>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="18"/>
+      <c r="A44" s="21"/>
       <c r="B44" s="3">
         <v>3</v>
       </c>
@@ -4162,7 +4163,7 @@
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" s="18"/>
+      <c r="A45" s="21"/>
       <c r="B45" s="3">
         <v>4</v>
       </c>
@@ -4228,7 +4229,7 @@
       </c>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A46" s="18"/>
+      <c r="A46" s="21"/>
       <c r="B46" s="3">
         <v>5</v>
       </c>
@@ -4294,7 +4295,7 @@
       </c>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="19" t="s">
+      <c r="A47" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B47" s="3">
@@ -4362,7 +4363,7 @@
       </c>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="20"/>
+      <c r="A48" s="23"/>
       <c r="B48" s="4">
         <v>7</v>
       </c>
@@ -4428,7 +4429,7 @@
       </c>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A49" s="21"/>
+      <c r="A49" s="24"/>
       <c r="B49" s="4">
         <v>8</v>
       </c>
@@ -4494,28 +4495,28 @@
       </c>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C52" s="22" t="s">
+      <c r="C52" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="23"/>
-      <c r="E52" s="23"/>
-      <c r="F52" s="23"/>
-      <c r="G52" s="23"/>
-      <c r="H52" s="23"/>
-      <c r="I52" s="23"/>
-      <c r="J52" s="23"/>
-      <c r="K52" s="23"/>
-      <c r="L52" s="23"/>
-      <c r="M52" s="23"/>
-      <c r="N52" s="23"/>
-      <c r="O52" s="23"/>
-      <c r="P52" s="23"/>
-      <c r="Q52" s="23"/>
-      <c r="R52" s="23"/>
-      <c r="S52" s="23"/>
-      <c r="T52" s="23"/>
-      <c r="U52" s="23"/>
-      <c r="V52" s="24"/>
+      <c r="D52" s="19"/>
+      <c r="E52" s="19"/>
+      <c r="F52" s="19"/>
+      <c r="G52" s="19"/>
+      <c r="H52" s="19"/>
+      <c r="I52" s="19"/>
+      <c r="J52" s="19"/>
+      <c r="K52" s="19"/>
+      <c r="L52" s="19"/>
+      <c r="M52" s="19"/>
+      <c r="N52" s="19"/>
+      <c r="O52" s="19"/>
+      <c r="P52" s="19"/>
+      <c r="Q52" s="19"/>
+      <c r="R52" s="19"/>
+      <c r="S52" s="19"/>
+      <c r="T52" s="19"/>
+      <c r="U52" s="19"/>
+      <c r="V52" s="20"/>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B53" s="1"/>
@@ -4581,75 +4582,75 @@
       </c>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A54" s="18" t="s">
+      <c r="A54" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="3">
         <v>1</v>
       </c>
       <c r="C54" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J54" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="L54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="M54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="P54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="S54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="T54" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="U54" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="H54" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="I54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J54" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="K54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="L54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="M54" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="N54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="O54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="P54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q54" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="R54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="S54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="T54" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="U54" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="V54" s="1" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A55" s="18"/>
+      <c r="A55" s="21"/>
       <c r="B55" s="3">
         <v>2</v>
       </c>
@@ -4657,65 +4658,65 @@
         <v>73</v>
       </c>
       <c r="D55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="L55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="M55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="P55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="S55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="T55" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="U55" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="H55" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="I55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K55" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="L55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="M55" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="N55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="O55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="P55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q55" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="R55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="S55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="T55" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="U55" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="V55" s="1" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A56" s="18"/>
+      <c r="A56" s="21"/>
       <c r="B56" s="3">
         <v>3</v>
       </c>
@@ -4726,62 +4727,62 @@
         <v>73</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="L56" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="M56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N56" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="O56" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="P56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="S56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="T56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="U56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="V56" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="F56" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="H56" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I56" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J56" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K56" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="L56" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="M56" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="N56" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="O56" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="P56" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q56" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="R56" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="S56" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="T56" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="U56" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="V56" s="1" t="s">
-        <v>73</v>
-      </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" s="18"/>
+      <c r="A57" s="21"/>
       <c r="B57" s="3">
         <v>4</v>
       </c>
@@ -4795,16 +4796,16 @@
         <v>73</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H57" s="1" t="s">
         <v>73</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="J57" s="1" t="s">
         <v>73</v>
@@ -4813,16 +4814,16 @@
         <v>73</v>
       </c>
       <c r="L57" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="M57" s="1" t="s">
         <v>73</v>
       </c>
       <c r="N57" s="1" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="O57" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="P57" s="1" t="s">
         <v>73</v>
@@ -4831,7 +4832,7 @@
         <v>73</v>
       </c>
       <c r="R57" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="S57" s="1" t="s">
         <v>73</v>
@@ -4840,14 +4841,14 @@
         <v>73</v>
       </c>
       <c r="U57" s="1" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="V57" s="1" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A58" s="18"/>
+      <c r="A58" s="21"/>
       <c r="B58" s="3">
         <v>5</v>
       </c>
@@ -4870,7 +4871,7 @@
         <v>73</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="J58" s="1" t="s">
         <v>73</v>
@@ -4879,28 +4880,28 @@
         <v>73</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="M58" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
       <c r="O58" s="1" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
       <c r="P58" s="1" t="s">
         <v>73</v>
       </c>
       <c r="Q58" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R58" s="1" t="s">
         <v>73</v>
       </c>
       <c r="S58" s="1" t="s">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="T58" s="1" t="s">
         <v>73</v>
@@ -4913,7 +4914,7 @@
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="19" t="s">
+      <c r="A59" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B59" s="3">
@@ -4981,7 +4982,7 @@
       </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="20"/>
+      <c r="A60" s="23"/>
       <c r="B60" s="4">
         <v>7</v>
       </c>
@@ -5047,7 +5048,7 @@
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="21"/>
+      <c r="A61" s="24"/>
       <c r="B61" s="4">
         <v>8</v>
       </c>
@@ -5113,28 +5114,28 @@
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C64" s="22" t="s">
+      <c r="C64" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D64" s="23"/>
-      <c r="E64" s="23"/>
-      <c r="F64" s="23"/>
-      <c r="G64" s="23"/>
-      <c r="H64" s="23"/>
-      <c r="I64" s="23"/>
-      <c r="J64" s="23"/>
-      <c r="K64" s="23"/>
-      <c r="L64" s="23"/>
-      <c r="M64" s="23"/>
-      <c r="N64" s="23"/>
-      <c r="O64" s="23"/>
-      <c r="P64" s="23"/>
-      <c r="Q64" s="23"/>
-      <c r="R64" s="23"/>
-      <c r="S64" s="23"/>
-      <c r="T64" s="23"/>
-      <c r="U64" s="23"/>
-      <c r="V64" s="24"/>
+      <c r="D64" s="19"/>
+      <c r="E64" s="19"/>
+      <c r="F64" s="19"/>
+      <c r="G64" s="19"/>
+      <c r="H64" s="19"/>
+      <c r="I64" s="19"/>
+      <c r="J64" s="19"/>
+      <c r="K64" s="19"/>
+      <c r="L64" s="19"/>
+      <c r="M64" s="19"/>
+      <c r="N64" s="19"/>
+      <c r="O64" s="19"/>
+      <c r="P64" s="19"/>
+      <c r="Q64" s="19"/>
+      <c r="R64" s="19"/>
+      <c r="S64" s="19"/>
+      <c r="T64" s="19"/>
+      <c r="U64" s="19"/>
+      <c r="V64" s="20"/>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B65" s="1"/>
@@ -5200,7 +5201,7 @@
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="18" t="s">
+      <c r="A66" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B66" s="3">
@@ -5216,59 +5217,59 @@
         <v>73</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="G66" s="1" t="s">
         <v>73</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="M66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="P66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="R66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="S66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="T66" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="U66" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="V66" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="J66" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K66" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="L66" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="M66" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="N66" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="O66" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="P66" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q66" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="R66" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="S66" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="T66" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="U66" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="V66" s="1" t="s">
-        <v>73</v>
-      </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="18"/>
+      <c r="A67" s="21"/>
       <c r="B67" s="3">
         <v>2</v>
       </c>
@@ -5282,13 +5283,13 @@
         <v>73</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G67" s="1" t="s">
         <v>73</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I67" s="1" t="s">
         <v>73</v>
@@ -5300,10 +5301,10 @@
         <v>73</v>
       </c>
       <c r="L67" s="1" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
       <c r="M67" s="1" t="s">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="N67" s="1" t="s">
         <v>73</v>
@@ -5321,20 +5322,20 @@
         <v>73</v>
       </c>
       <c r="S67" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="T67" s="1" t="s">
         <v>73</v>
       </c>
       <c r="U67" s="1" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="V67" s="1" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" s="18"/>
+      <c r="A68" s="21"/>
       <c r="B68" s="3">
         <v>3</v>
       </c>
@@ -5348,16 +5349,16 @@
         <v>73</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="H68" s="1" t="s">
         <v>73</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="J68" s="1" t="s">
         <v>73</v>
@@ -5366,22 +5367,22 @@
         <v>73</v>
       </c>
       <c r="L68" s="1" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
       <c r="M68" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="O68" s="1" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="P68" s="1" t="s">
         <v>73</v>
       </c>
       <c r="Q68" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R68" s="1" t="s">
         <v>73</v>
@@ -5400,7 +5401,7 @@
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="18"/>
+      <c r="A69" s="21"/>
       <c r="B69" s="3">
         <v>4</v>
       </c>
@@ -5417,7 +5418,7 @@
         <v>73</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H69" s="1" t="s">
         <v>73</v>
@@ -5435,19 +5436,19 @@
         <v>73</v>
       </c>
       <c r="M69" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="O69" s="1" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="P69" s="1" t="s">
         <v>73</v>
       </c>
       <c r="Q69" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R69" s="1" t="s">
         <v>73</v>
@@ -5466,7 +5467,7 @@
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="18"/>
+      <c r="A70" s="21"/>
       <c r="B70" s="3">
         <v>5</v>
       </c>
@@ -5483,13 +5484,13 @@
         <v>73</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="H70" s="1" t="s">
         <v>73</v>
       </c>
       <c r="I70" s="1" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="J70" s="1" t="s">
         <v>73</v>
@@ -5504,7 +5505,7 @@
         <v>73</v>
       </c>
       <c r="N70" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="O70" s="1" t="s">
         <v>73</v>
@@ -5516,7 +5517,7 @@
         <v>73</v>
       </c>
       <c r="R70" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="S70" s="1" t="s">
         <v>73</v>
@@ -5532,7 +5533,7 @@
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A71" s="19" t="s">
+      <c r="A71" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B71" s="3">
@@ -5600,7 +5601,7 @@
       </c>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="20"/>
+      <c r="A72" s="23"/>
       <c r="B72" s="4">
         <v>7</v>
       </c>
@@ -5666,7 +5667,7 @@
       </c>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" s="21"/>
+      <c r="A73" s="24"/>
       <c r="B73" s="4">
         <v>8</v>
       </c>
@@ -5733,16 +5734,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C4:V4"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="C16:V16"/>
-    <mergeCell ref="A18:A22"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C28:V28"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="C64:V64"/>
     <mergeCell ref="A66:A70"/>
     <mergeCell ref="A71:A73"/>
     <mergeCell ref="C40:V40"/>
@@ -5751,6 +5742,16 @@
     <mergeCell ref="C52:V52"/>
     <mergeCell ref="A54:A58"/>
     <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C28:V28"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="C64:V64"/>
+    <mergeCell ref="C4:V4"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="C16:V16"/>
+    <mergeCell ref="A18:A22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
having relax time at the noon
</commit_message>
<xml_diff>
--- a/src/excel_resources/excel_data.xlsx
+++ b/src/excel_resources/excel_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F95676F4-FDF9-4DED-9845-F83B0BC78DE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9343F26A-BD00-4C7C-B6DC-63003231AC6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4087" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7927" uniqueCount="108">
   <si>
     <t>10A1</t>
   </si>
@@ -552,6 +552,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -563,15 +572,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -967,7 +967,7 @@
         <v>CD Văn</v>
       </c>
       <c r="D8" s="13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" s="13">
         <v>35</v>
@@ -2169,28 +2169,28 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="23"/>
-      <c r="R4" s="23"/>
-      <c r="S4" s="23"/>
-      <c r="T4" s="23"/>
-      <c r="U4" s="23"/>
-      <c r="V4" s="24"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="20"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
@@ -2256,7 +2256,7 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="3">
@@ -2324,7 +2324,7 @@
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A7" s="18"/>
+      <c r="A7" s="21"/>
       <c r="B7" s="3">
         <v>2</v>
       </c>
@@ -2390,7 +2390,7 @@
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A8" s="18"/>
+      <c r="A8" s="21"/>
       <c r="B8" s="3">
         <v>3</v>
       </c>
@@ -2456,7 +2456,7 @@
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A9" s="18"/>
+      <c r="A9" s="21"/>
       <c r="B9" s="3">
         <v>4</v>
       </c>
@@ -2522,7 +2522,7 @@
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A10" s="18"/>
+      <c r="A10" s="21"/>
       <c r="B10" s="3">
         <v>5</v>
       </c>
@@ -2588,7 +2588,7 @@
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="3">
@@ -2656,7 +2656,7 @@
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="20"/>
+      <c r="A12" s="23"/>
       <c r="B12" s="4">
         <v>7</v>
       </c>
@@ -2722,7 +2722,7 @@
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A13" s="21"/>
+      <c r="A13" s="24"/>
       <c r="B13" s="4">
         <v>8</v>
       </c>
@@ -2788,28 +2788,28 @@
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
-      <c r="P16" s="23"/>
-      <c r="Q16" s="23"/>
-      <c r="R16" s="23"/>
-      <c r="S16" s="23"/>
-      <c r="T16" s="23"/>
-      <c r="U16" s="23"/>
-      <c r="V16" s="24"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
+      <c r="O16" s="19"/>
+      <c r="P16" s="19"/>
+      <c r="Q16" s="19"/>
+      <c r="R16" s="19"/>
+      <c r="S16" s="19"/>
+      <c r="T16" s="19"/>
+      <c r="U16" s="19"/>
+      <c r="V16" s="20"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -2875,7 +2875,7 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="3">
@@ -2943,7 +2943,7 @@
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A19" s="18"/>
+      <c r="A19" s="21"/>
       <c r="B19" s="3">
         <v>2</v>
       </c>
@@ -3009,7 +3009,7 @@
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A20" s="18"/>
+      <c r="A20" s="21"/>
       <c r="B20" s="3">
         <v>3</v>
       </c>
@@ -3075,7 +3075,7 @@
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A21" s="18"/>
+      <c r="A21" s="21"/>
       <c r="B21" s="3">
         <v>4</v>
       </c>
@@ -3141,7 +3141,7 @@
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A22" s="18"/>
+      <c r="A22" s="21"/>
       <c r="B22" s="3">
         <v>5</v>
       </c>
@@ -3207,7 +3207,7 @@
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="3">
@@ -3275,7 +3275,7 @@
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A24" s="20"/>
+      <c r="A24" s="23"/>
       <c r="B24" s="4">
         <v>7</v>
       </c>
@@ -3316,7 +3316,7 @@
         <v>72</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>72</v>
+        <v>105</v>
       </c>
       <c r="P24" s="1" t="s">
         <v>72</v>
@@ -3341,7 +3341,7 @@
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A25" s="21"/>
+      <c r="A25" s="24"/>
       <c r="B25" s="4">
         <v>8</v>
       </c>
@@ -3407,28 +3407,28 @@
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="23"/>
-      <c r="K28" s="23"/>
-      <c r="L28" s="23"/>
-      <c r="M28" s="23"/>
-      <c r="N28" s="23"/>
-      <c r="O28" s="23"/>
-      <c r="P28" s="23"/>
-      <c r="Q28" s="23"/>
-      <c r="R28" s="23"/>
-      <c r="S28" s="23"/>
-      <c r="T28" s="23"/>
-      <c r="U28" s="23"/>
-      <c r="V28" s="24"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="19"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="19"/>
+      <c r="N28" s="19"/>
+      <c r="O28" s="19"/>
+      <c r="P28" s="19"/>
+      <c r="Q28" s="19"/>
+      <c r="R28" s="19"/>
+      <c r="S28" s="19"/>
+      <c r="T28" s="19"/>
+      <c r="U28" s="19"/>
+      <c r="V28" s="20"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B29" s="1"/>
@@ -3494,7 +3494,7 @@
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="3">
@@ -3562,7 +3562,7 @@
       </c>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A31" s="18"/>
+      <c r="A31" s="21"/>
       <c r="B31" s="3">
         <v>2</v>
       </c>
@@ -3628,7 +3628,7 @@
       </c>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A32" s="18"/>
+      <c r="A32" s="21"/>
       <c r="B32" s="3">
         <v>3</v>
       </c>
@@ -3694,7 +3694,7 @@
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="18"/>
+      <c r="A33" s="21"/>
       <c r="B33" s="3">
         <v>4</v>
       </c>
@@ -3760,7 +3760,7 @@
       </c>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" s="18"/>
+      <c r="A34" s="21"/>
       <c r="B34" s="3">
         <v>5</v>
       </c>
@@ -3826,7 +3826,7 @@
       </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="3">
@@ -3894,7 +3894,7 @@
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="20"/>
+      <c r="A36" s="23"/>
       <c r="B36" s="4">
         <v>7</v>
       </c>
@@ -3960,7 +3960,7 @@
       </c>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="21"/>
+      <c r="A37" s="24"/>
       <c r="B37" s="4">
         <v>8</v>
       </c>
@@ -4026,28 +4026,28 @@
       </c>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C40" s="22" t="s">
+      <c r="C40" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="23"/>
-      <c r="E40" s="23"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
-      <c r="H40" s="23"/>
-      <c r="I40" s="23"/>
-      <c r="J40" s="23"/>
-      <c r="K40" s="23"/>
-      <c r="L40" s="23"/>
-      <c r="M40" s="23"/>
-      <c r="N40" s="23"/>
-      <c r="O40" s="23"/>
-      <c r="P40" s="23"/>
-      <c r="Q40" s="23"/>
-      <c r="R40" s="23"/>
-      <c r="S40" s="23"/>
-      <c r="T40" s="23"/>
-      <c r="U40" s="23"/>
-      <c r="V40" s="24"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="19"/>
+      <c r="H40" s="19"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="19"/>
+      <c r="K40" s="19"/>
+      <c r="L40" s="19"/>
+      <c r="M40" s="19"/>
+      <c r="N40" s="19"/>
+      <c r="O40" s="19"/>
+      <c r="P40" s="19"/>
+      <c r="Q40" s="19"/>
+      <c r="R40" s="19"/>
+      <c r="S40" s="19"/>
+      <c r="T40" s="19"/>
+      <c r="U40" s="19"/>
+      <c r="V40" s="20"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B41" s="1"/>
@@ -4113,7 +4113,7 @@
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="18" t="s">
+      <c r="A42" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="3">
@@ -4181,7 +4181,7 @@
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="18"/>
+      <c r="A43" s="21"/>
       <c r="B43" s="3">
         <v>2</v>
       </c>
@@ -4247,7 +4247,7 @@
       </c>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="18"/>
+      <c r="A44" s="21"/>
       <c r="B44" s="3">
         <v>3</v>
       </c>
@@ -4313,7 +4313,7 @@
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" s="18"/>
+      <c r="A45" s="21"/>
       <c r="B45" s="3">
         <v>4</v>
       </c>
@@ -4379,7 +4379,7 @@
       </c>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A46" s="18"/>
+      <c r="A46" s="21"/>
       <c r="B46" s="3">
         <v>5</v>
       </c>
@@ -4445,7 +4445,7 @@
       </c>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="19" t="s">
+      <c r="A47" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B47" s="3">
@@ -4513,7 +4513,7 @@
       </c>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="20"/>
+      <c r="A48" s="23"/>
       <c r="B48" s="4">
         <v>7</v>
       </c>
@@ -4579,7 +4579,7 @@
       </c>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A49" s="21"/>
+      <c r="A49" s="24"/>
       <c r="B49" s="4">
         <v>8</v>
       </c>
@@ -4645,28 +4645,28 @@
       </c>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C52" s="22" t="s">
+      <c r="C52" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="23"/>
-      <c r="E52" s="23"/>
-      <c r="F52" s="23"/>
-      <c r="G52" s="23"/>
-      <c r="H52" s="23"/>
-      <c r="I52" s="23"/>
-      <c r="J52" s="23"/>
-      <c r="K52" s="23"/>
-      <c r="L52" s="23"/>
-      <c r="M52" s="23"/>
-      <c r="N52" s="23"/>
-      <c r="O52" s="23"/>
-      <c r="P52" s="23"/>
-      <c r="Q52" s="23"/>
-      <c r="R52" s="23"/>
-      <c r="S52" s="23"/>
-      <c r="T52" s="23"/>
-      <c r="U52" s="23"/>
-      <c r="V52" s="24"/>
+      <c r="D52" s="19"/>
+      <c r="E52" s="19"/>
+      <c r="F52" s="19"/>
+      <c r="G52" s="19"/>
+      <c r="H52" s="19"/>
+      <c r="I52" s="19"/>
+      <c r="J52" s="19"/>
+      <c r="K52" s="19"/>
+      <c r="L52" s="19"/>
+      <c r="M52" s="19"/>
+      <c r="N52" s="19"/>
+      <c r="O52" s="19"/>
+      <c r="P52" s="19"/>
+      <c r="Q52" s="19"/>
+      <c r="R52" s="19"/>
+      <c r="S52" s="19"/>
+      <c r="T52" s="19"/>
+      <c r="U52" s="19"/>
+      <c r="V52" s="20"/>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B53" s="1"/>
@@ -4732,7 +4732,7 @@
       </c>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A54" s="18" t="s">
+      <c r="A54" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="3">
@@ -4800,7 +4800,7 @@
       </c>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A55" s="18"/>
+      <c r="A55" s="21"/>
       <c r="B55" s="3">
         <v>2</v>
       </c>
@@ -4866,7 +4866,7 @@
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A56" s="18"/>
+      <c r="A56" s="21"/>
       <c r="B56" s="3">
         <v>3</v>
       </c>
@@ -4932,7 +4932,7 @@
       </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" s="18"/>
+      <c r="A57" s="21"/>
       <c r="B57" s="3">
         <v>4</v>
       </c>
@@ -4998,7 +4998,7 @@
       </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A58" s="18"/>
+      <c r="A58" s="21"/>
       <c r="B58" s="3">
         <v>5</v>
       </c>
@@ -5064,7 +5064,7 @@
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="19" t="s">
+      <c r="A59" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B59" s="3">
@@ -5132,7 +5132,7 @@
       </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="20"/>
+      <c r="A60" s="23"/>
       <c r="B60" s="4">
         <v>7</v>
       </c>
@@ -5198,7 +5198,7 @@
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="21"/>
+      <c r="A61" s="24"/>
       <c r="B61" s="4">
         <v>8</v>
       </c>
@@ -5264,28 +5264,28 @@
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C64" s="22" t="s">
+      <c r="C64" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D64" s="23"/>
-      <c r="E64" s="23"/>
-      <c r="F64" s="23"/>
-      <c r="G64" s="23"/>
-      <c r="H64" s="23"/>
-      <c r="I64" s="23"/>
-      <c r="J64" s="23"/>
-      <c r="K64" s="23"/>
-      <c r="L64" s="23"/>
-      <c r="M64" s="23"/>
-      <c r="N64" s="23"/>
-      <c r="O64" s="23"/>
-      <c r="P64" s="23"/>
-      <c r="Q64" s="23"/>
-      <c r="R64" s="23"/>
-      <c r="S64" s="23"/>
-      <c r="T64" s="23"/>
-      <c r="U64" s="23"/>
-      <c r="V64" s="24"/>
+      <c r="D64" s="19"/>
+      <c r="E64" s="19"/>
+      <c r="F64" s="19"/>
+      <c r="G64" s="19"/>
+      <c r="H64" s="19"/>
+      <c r="I64" s="19"/>
+      <c r="J64" s="19"/>
+      <c r="K64" s="19"/>
+      <c r="L64" s="19"/>
+      <c r="M64" s="19"/>
+      <c r="N64" s="19"/>
+      <c r="O64" s="19"/>
+      <c r="P64" s="19"/>
+      <c r="Q64" s="19"/>
+      <c r="R64" s="19"/>
+      <c r="S64" s="19"/>
+      <c r="T64" s="19"/>
+      <c r="U64" s="19"/>
+      <c r="V64" s="20"/>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B65" s="1"/>
@@ -5351,7 +5351,7 @@
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="18" t="s">
+      <c r="A66" s="21" t="s">
         <v>20</v>
       </c>
       <c r="B66" s="3">
@@ -5419,7 +5419,7 @@
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="18"/>
+      <c r="A67" s="21"/>
       <c r="B67" s="3">
         <v>2</v>
       </c>
@@ -5460,7 +5460,7 @@
         <v>72</v>
       </c>
       <c r="O67" s="1" t="s">
-        <v>72</v>
+        <v>105</v>
       </c>
       <c r="P67" s="1" t="s">
         <v>72</v>
@@ -5485,7 +5485,7 @@
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" s="18"/>
+      <c r="A68" s="21"/>
       <c r="B68" s="3">
         <v>3</v>
       </c>
@@ -5551,7 +5551,7 @@
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="18"/>
+      <c r="A69" s="21"/>
       <c r="B69" s="3">
         <v>4</v>
       </c>
@@ -5617,7 +5617,7 @@
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="18"/>
+      <c r="A70" s="21"/>
       <c r="B70" s="3">
         <v>5</v>
       </c>
@@ -5683,7 +5683,7 @@
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A71" s="19" t="s">
+      <c r="A71" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B71" s="3">
@@ -5751,7 +5751,7 @@
       </c>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="20"/>
+      <c r="A72" s="23"/>
       <c r="B72" s="4">
         <v>7</v>
       </c>
@@ -5817,7 +5817,7 @@
       </c>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" s="21"/>
+      <c r="A73" s="24"/>
       <c r="B73" s="4">
         <v>8</v>
       </c>
@@ -5884,16 +5884,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C4:V4"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="C16:V16"/>
-    <mergeCell ref="A18:A22"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C28:V28"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="C64:V64"/>
     <mergeCell ref="A66:A70"/>
     <mergeCell ref="A71:A73"/>
     <mergeCell ref="C40:V40"/>
@@ -5902,6 +5892,16 @@
     <mergeCell ref="C52:V52"/>
     <mergeCell ref="A54:A58"/>
     <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C28:V28"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="C64:V64"/>
+    <mergeCell ref="C4:V4"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="C16:V16"/>
+    <mergeCell ref="A18:A22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
renovate distribution lessons equally function
</commit_message>
<xml_diff>
--- a/src/excel_resources/excel_data.xlsx
+++ b/src/excel_resources/excel_data.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AC59CBD-F45D-4193-AA5A-7290932A14D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A09B352-3BA8-4B37-B27C-08D183ABD690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10807" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1207" uniqueCount="108">
   <si>
     <t>10A1</t>
   </si>
@@ -356,7 +356,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -552,15 +551,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -572,6 +562,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -856,25 +855,25 @@
   <dimension ref="A5:U124"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="28.08984375"/>
-    <col min="2" max="2" customWidth="true" width="63.08984375"/>
-    <col min="3" max="3" customWidth="true" width="20.1796875"/>
-    <col min="4" max="4" customWidth="true" width="16.36328125"/>
-    <col min="5" max="5" customWidth="true" width="15.26953125"/>
-    <col min="6" max="6" customWidth="true" width="22.7265625"/>
-    <col min="7" max="7" customWidth="true" width="21.54296875"/>
-    <col min="8" max="8" customWidth="true" width="20.36328125"/>
-    <col min="9" max="9" customWidth="true" width="26.453125"/>
-    <col min="10" max="10" customWidth="true" width="22.81640625"/>
-    <col min="11" max="11" customWidth="true" width="23.36328125"/>
-    <col min="12" max="12" customWidth="true" width="12.7265625"/>
-    <col min="13" max="13" customWidth="true" width="19.1796875"/>
-    <col min="14" max="14" customWidth="true" width="16.08984375"/>
-    <col min="15" max="15" customWidth="true" width="16.1796875"/>
-    <col min="16" max="16" customWidth="true" width="10.90625"/>
-    <col min="17" max="17" customWidth="true" width="13.54296875"/>
-    <col min="20" max="20" customWidth="true" width="17.08984375"/>
-    <col min="21" max="21" customWidth="true" width="9.90625"/>
+    <col min="1" max="1" width="28.08984375" customWidth="1"/>
+    <col min="2" max="2" width="63.08984375" customWidth="1"/>
+    <col min="3" max="3" width="20.1796875" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" customWidth="1"/>
+    <col min="5" max="5" width="15.26953125" customWidth="1"/>
+    <col min="6" max="6" width="22.7265625" customWidth="1"/>
+    <col min="7" max="7" width="21.54296875" customWidth="1"/>
+    <col min="8" max="8" width="20.36328125" customWidth="1"/>
+    <col min="9" max="9" width="26.453125" customWidth="1"/>
+    <col min="10" max="10" width="22.81640625" customWidth="1"/>
+    <col min="11" max="11" width="23.36328125" customWidth="1"/>
+    <col min="12" max="12" width="12.7265625" customWidth="1"/>
+    <col min="13" max="13" width="19.1796875" customWidth="1"/>
+    <col min="14" max="14" width="16.08984375" customWidth="1"/>
+    <col min="15" max="15" width="16.1796875" customWidth="1"/>
+    <col min="16" max="16" width="10.90625" customWidth="1"/>
+    <col min="17" max="17" width="13.54296875" customWidth="1"/>
+    <col min="20" max="20" width="17.08984375" customWidth="1"/>
+    <col min="21" max="21" width="9.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
@@ -2160,37 +2159,37 @@
   <dimension ref="A4:V73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="10" max="10" customWidth="true" width="24.90625"/>
-    <col min="11" max="11" customWidth="true" width="17.90625"/>
-    <col min="15" max="15" customWidth="true" width="17.453125"/>
-    <col min="17" max="17" customWidth="true" width="19.6328125"/>
-    <col min="18" max="18" customWidth="true" width="24.36328125"/>
-    <col min="19" max="19" customWidth="true" width="23.0"/>
+    <col min="10" max="10" width="24.90625" customWidth="1"/>
+    <col min="11" max="11" width="17.90625" customWidth="1"/>
+    <col min="15" max="15" width="17.453125" customWidth="1"/>
+    <col min="17" max="17" width="19.6328125" customWidth="1"/>
+    <col min="18" max="18" width="24.36328125" customWidth="1"/>
+    <col min="19" max="19" width="23" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="19"/>
-      <c r="U4" s="19"/>
-      <c r="V4" s="20"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="23"/>
+      <c r="T4" s="23"/>
+      <c r="U4" s="23"/>
+      <c r="V4" s="24"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
@@ -2256,7 +2255,7 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="3">
@@ -2324,7 +2323,7 @@
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A7" s="21"/>
+      <c r="A7" s="18"/>
       <c r="B7" s="3">
         <v>2</v>
       </c>
@@ -2390,7 +2389,7 @@
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A8" s="21"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="3">
         <v>3</v>
       </c>
@@ -2456,7 +2455,7 @@
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A9" s="21"/>
+      <c r="A9" s="18"/>
       <c r="B9" s="3">
         <v>4</v>
       </c>
@@ -2522,7 +2521,7 @@
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A10" s="21"/>
+      <c r="A10" s="18"/>
       <c r="B10" s="3">
         <v>5</v>
       </c>
@@ -2588,7 +2587,7 @@
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="3">
@@ -2610,7 +2609,7 @@
         <v>72</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>72</v>
@@ -2656,7 +2655,7 @@
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="23"/>
+      <c r="A12" s="20"/>
       <c r="B12" s="4">
         <v>7</v>
       </c>
@@ -2697,7 +2696,7 @@
         <v>105</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="P12" s="1" t="s">
         <v>72</v>
@@ -2722,7 +2721,7 @@
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A13" s="24"/>
+      <c r="A13" s="21"/>
       <c r="B13" s="4">
         <v>8</v>
       </c>
@@ -2788,28 +2787,28 @@
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
-      <c r="L16" s="19"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="19"/>
-      <c r="O16" s="19"/>
-      <c r="P16" s="19"/>
-      <c r="Q16" s="19"/>
-      <c r="R16" s="19"/>
-      <c r="S16" s="19"/>
-      <c r="T16" s="19"/>
-      <c r="U16" s="19"/>
-      <c r="V16" s="20"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="23"/>
+      <c r="N16" s="23"/>
+      <c r="O16" s="23"/>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="23"/>
+      <c r="R16" s="23"/>
+      <c r="S16" s="23"/>
+      <c r="T16" s="23"/>
+      <c r="U16" s="23"/>
+      <c r="V16" s="24"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -2875,7 +2874,7 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="3">
@@ -2943,7 +2942,7 @@
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A19" s="21"/>
+      <c r="A19" s="18"/>
       <c r="B19" s="3">
         <v>2</v>
       </c>
@@ -3009,7 +3008,7 @@
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A20" s="21"/>
+      <c r="A20" s="18"/>
       <c r="B20" s="3">
         <v>3</v>
       </c>
@@ -3075,7 +3074,7 @@
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A21" s="21"/>
+      <c r="A21" s="18"/>
       <c r="B21" s="3">
         <v>4</v>
       </c>
@@ -3141,7 +3140,7 @@
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A22" s="21"/>
+      <c r="A22" s="18"/>
       <c r="B22" s="3">
         <v>5</v>
       </c>
@@ -3207,7 +3206,7 @@
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="3">
@@ -3229,7 +3228,7 @@
         <v>72</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>72</v>
+        <v>104</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>106</v>
@@ -3275,7 +3274,7 @@
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A24" s="23"/>
+      <c r="A24" s="20"/>
       <c r="B24" s="4">
         <v>7</v>
       </c>
@@ -3341,7 +3340,7 @@
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A25" s="24"/>
+      <c r="A25" s="21"/>
       <c r="B25" s="4">
         <v>8</v>
       </c>
@@ -3407,28 +3406,28 @@
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
-      <c r="L28" s="19"/>
-      <c r="M28" s="19"/>
-      <c r="N28" s="19"/>
-      <c r="O28" s="19"/>
-      <c r="P28" s="19"/>
-      <c r="Q28" s="19"/>
-      <c r="R28" s="19"/>
-      <c r="S28" s="19"/>
-      <c r="T28" s="19"/>
-      <c r="U28" s="19"/>
-      <c r="V28" s="20"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="23"/>
+      <c r="I28" s="23"/>
+      <c r="J28" s="23"/>
+      <c r="K28" s="23"/>
+      <c r="L28" s="23"/>
+      <c r="M28" s="23"/>
+      <c r="N28" s="23"/>
+      <c r="O28" s="23"/>
+      <c r="P28" s="23"/>
+      <c r="Q28" s="23"/>
+      <c r="R28" s="23"/>
+      <c r="S28" s="23"/>
+      <c r="T28" s="23"/>
+      <c r="U28" s="23"/>
+      <c r="V28" s="24"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B29" s="1"/>
@@ -3494,7 +3493,7 @@
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="21" t="s">
+      <c r="A30" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="3">
@@ -3562,7 +3561,7 @@
       </c>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A31" s="21"/>
+      <c r="A31" s="18"/>
       <c r="B31" s="3">
         <v>2</v>
       </c>
@@ -3628,7 +3627,7 @@
       </c>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A32" s="21"/>
+      <c r="A32" s="18"/>
       <c r="B32" s="3">
         <v>3</v>
       </c>
@@ -3694,7 +3693,7 @@
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="21"/>
+      <c r="A33" s="18"/>
       <c r="B33" s="3">
         <v>4</v>
       </c>
@@ -3760,7 +3759,7 @@
       </c>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" s="21"/>
+      <c r="A34" s="18"/>
       <c r="B34" s="3">
         <v>5</v>
       </c>
@@ -3826,7 +3825,7 @@
       </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="3">
@@ -3860,7 +3859,7 @@
         <v>72</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="M35" s="1" t="s">
         <v>72</v>
@@ -3894,7 +3893,7 @@
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="23"/>
+      <c r="A36" s="20"/>
       <c r="B36" s="4">
         <v>7</v>
       </c>
@@ -3960,7 +3959,7 @@
       </c>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="24"/>
+      <c r="A37" s="21"/>
       <c r="B37" s="4">
         <v>8</v>
       </c>
@@ -4026,28 +4025,28 @@
       </c>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C40" s="18" t="s">
+      <c r="C40" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="19"/>
-      <c r="E40" s="19"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="19"/>
-      <c r="H40" s="19"/>
-      <c r="I40" s="19"/>
-      <c r="J40" s="19"/>
-      <c r="K40" s="19"/>
-      <c r="L40" s="19"/>
-      <c r="M40" s="19"/>
-      <c r="N40" s="19"/>
-      <c r="O40" s="19"/>
-      <c r="P40" s="19"/>
-      <c r="Q40" s="19"/>
-      <c r="R40" s="19"/>
-      <c r="S40" s="19"/>
-      <c r="T40" s="19"/>
-      <c r="U40" s="19"/>
-      <c r="V40" s="20"/>
+      <c r="D40" s="23"/>
+      <c r="E40" s="23"/>
+      <c r="F40" s="23"/>
+      <c r="G40" s="23"/>
+      <c r="H40" s="23"/>
+      <c r="I40" s="23"/>
+      <c r="J40" s="23"/>
+      <c r="K40" s="23"/>
+      <c r="L40" s="23"/>
+      <c r="M40" s="23"/>
+      <c r="N40" s="23"/>
+      <c r="O40" s="23"/>
+      <c r="P40" s="23"/>
+      <c r="Q40" s="23"/>
+      <c r="R40" s="23"/>
+      <c r="S40" s="23"/>
+      <c r="T40" s="23"/>
+      <c r="U40" s="23"/>
+      <c r="V40" s="24"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B41" s="1"/>
@@ -4113,7 +4112,7 @@
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="21" t="s">
+      <c r="A42" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="3">
@@ -4181,7 +4180,7 @@
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="21"/>
+      <c r="A43" s="18"/>
       <c r="B43" s="3">
         <v>2</v>
       </c>
@@ -4247,7 +4246,7 @@
       </c>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="21"/>
+      <c r="A44" s="18"/>
       <c r="B44" s="3">
         <v>3</v>
       </c>
@@ -4313,7 +4312,7 @@
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" s="21"/>
+      <c r="A45" s="18"/>
       <c r="B45" s="3">
         <v>4</v>
       </c>
@@ -4379,7 +4378,7 @@
       </c>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A46" s="21"/>
+      <c r="A46" s="18"/>
       <c r="B46" s="3">
         <v>5</v>
       </c>
@@ -4445,7 +4444,7 @@
       </c>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="22" t="s">
+      <c r="A47" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B47" s="3">
@@ -4513,7 +4512,7 @@
       </c>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="23"/>
+      <c r="A48" s="20"/>
       <c r="B48" s="4">
         <v>7</v>
       </c>
@@ -4579,7 +4578,7 @@
       </c>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A49" s="24"/>
+      <c r="A49" s="21"/>
       <c r="B49" s="4">
         <v>8</v>
       </c>
@@ -4645,28 +4644,28 @@
       </c>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C52" s="18" t="s">
+      <c r="C52" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="19"/>
-      <c r="E52" s="19"/>
-      <c r="F52" s="19"/>
-      <c r="G52" s="19"/>
-      <c r="H52" s="19"/>
-      <c r="I52" s="19"/>
-      <c r="J52" s="19"/>
-      <c r="K52" s="19"/>
-      <c r="L52" s="19"/>
-      <c r="M52" s="19"/>
-      <c r="N52" s="19"/>
-      <c r="O52" s="19"/>
-      <c r="P52" s="19"/>
-      <c r="Q52" s="19"/>
-      <c r="R52" s="19"/>
-      <c r="S52" s="19"/>
-      <c r="T52" s="19"/>
-      <c r="U52" s="19"/>
-      <c r="V52" s="20"/>
+      <c r="D52" s="23"/>
+      <c r="E52" s="23"/>
+      <c r="F52" s="23"/>
+      <c r="G52" s="23"/>
+      <c r="H52" s="23"/>
+      <c r="I52" s="23"/>
+      <c r="J52" s="23"/>
+      <c r="K52" s="23"/>
+      <c r="L52" s="23"/>
+      <c r="M52" s="23"/>
+      <c r="N52" s="23"/>
+      <c r="O52" s="23"/>
+      <c r="P52" s="23"/>
+      <c r="Q52" s="23"/>
+      <c r="R52" s="23"/>
+      <c r="S52" s="23"/>
+      <c r="T52" s="23"/>
+      <c r="U52" s="23"/>
+      <c r="V52" s="24"/>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B53" s="1"/>
@@ -4732,7 +4731,7 @@
       </c>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A54" s="21" t="s">
+      <c r="A54" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="3">
@@ -4800,7 +4799,7 @@
       </c>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A55" s="21"/>
+      <c r="A55" s="18"/>
       <c r="B55" s="3">
         <v>2</v>
       </c>
@@ -4866,7 +4865,7 @@
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A56" s="21"/>
+      <c r="A56" s="18"/>
       <c r="B56" s="3">
         <v>3</v>
       </c>
@@ -4932,7 +4931,7 @@
       </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" s="21"/>
+      <c r="A57" s="18"/>
       <c r="B57" s="3">
         <v>4</v>
       </c>
@@ -4998,7 +4997,7 @@
       </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A58" s="21"/>
+      <c r="A58" s="18"/>
       <c r="B58" s="3">
         <v>5</v>
       </c>
@@ -5064,7 +5063,7 @@
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="22" t="s">
+      <c r="A59" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B59" s="3">
@@ -5098,7 +5097,7 @@
         <v>72</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>105</v>
+        <v>72</v>
       </c>
       <c r="M59" s="1" t="s">
         <v>72</v>
@@ -5132,7 +5131,7 @@
       </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="23"/>
+      <c r="A60" s="20"/>
       <c r="B60" s="4">
         <v>7</v>
       </c>
@@ -5198,7 +5197,7 @@
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="24"/>
+      <c r="A61" s="21"/>
       <c r="B61" s="4">
         <v>8</v>
       </c>
@@ -5264,28 +5263,28 @@
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C64" s="18" t="s">
+      <c r="C64" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="D64" s="19"/>
-      <c r="E64" s="19"/>
-      <c r="F64" s="19"/>
-      <c r="G64" s="19"/>
-      <c r="H64" s="19"/>
-      <c r="I64" s="19"/>
-      <c r="J64" s="19"/>
-      <c r="K64" s="19"/>
-      <c r="L64" s="19"/>
-      <c r="M64" s="19"/>
-      <c r="N64" s="19"/>
-      <c r="O64" s="19"/>
-      <c r="P64" s="19"/>
-      <c r="Q64" s="19"/>
-      <c r="R64" s="19"/>
-      <c r="S64" s="19"/>
-      <c r="T64" s="19"/>
-      <c r="U64" s="19"/>
-      <c r="V64" s="20"/>
+      <c r="D64" s="23"/>
+      <c r="E64" s="23"/>
+      <c r="F64" s="23"/>
+      <c r="G64" s="23"/>
+      <c r="H64" s="23"/>
+      <c r="I64" s="23"/>
+      <c r="J64" s="23"/>
+      <c r="K64" s="23"/>
+      <c r="L64" s="23"/>
+      <c r="M64" s="23"/>
+      <c r="N64" s="23"/>
+      <c r="O64" s="23"/>
+      <c r="P64" s="23"/>
+      <c r="Q64" s="23"/>
+      <c r="R64" s="23"/>
+      <c r="S64" s="23"/>
+      <c r="T64" s="23"/>
+      <c r="U64" s="23"/>
+      <c r="V64" s="24"/>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B65" s="1"/>
@@ -5351,7 +5350,7 @@
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="21" t="s">
+      <c r="A66" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B66" s="3">
@@ -5419,7 +5418,7 @@
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="21"/>
+      <c r="A67" s="18"/>
       <c r="B67" s="3">
         <v>2</v>
       </c>
@@ -5485,7 +5484,7 @@
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" s="21"/>
+      <c r="A68" s="18"/>
       <c r="B68" s="3">
         <v>3</v>
       </c>
@@ -5551,7 +5550,7 @@
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="21"/>
+      <c r="A69" s="18"/>
       <c r="B69" s="3">
         <v>4</v>
       </c>
@@ -5617,7 +5616,7 @@
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="21"/>
+      <c r="A70" s="18"/>
       <c r="B70" s="3">
         <v>5</v>
       </c>
@@ -5683,7 +5682,7 @@
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A71" s="22" t="s">
+      <c r="A71" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B71" s="3">
@@ -5717,7 +5716,7 @@
         <v>72</v>
       </c>
       <c r="L71" s="1" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="M71" s="1" t="s">
         <v>72</v>
@@ -5751,7 +5750,7 @@
       </c>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="23"/>
+      <c r="A72" s="20"/>
       <c r="B72" s="4">
         <v>7</v>
       </c>
@@ -5792,7 +5791,7 @@
         <v>72</v>
       </c>
       <c r="O72" s="1" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="P72" s="1" t="s">
         <v>72</v>
@@ -5817,7 +5816,7 @@
       </c>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" s="24"/>
+      <c r="A73" s="21"/>
       <c r="B73" s="4">
         <v>8</v>
       </c>
@@ -5884,6 +5883,16 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C4:V4"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="C16:V16"/>
+    <mergeCell ref="A18:A22"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C28:V28"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="C64:V64"/>
     <mergeCell ref="A66:A70"/>
     <mergeCell ref="A71:A73"/>
     <mergeCell ref="C40:V40"/>
@@ -5892,16 +5901,6 @@
     <mergeCell ref="C52:V52"/>
     <mergeCell ref="A54:A58"/>
     <mergeCell ref="A59:A61"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C28:V28"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="C64:V64"/>
-    <mergeCell ref="C4:V4"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="C16:V16"/>
-    <mergeCell ref="A18:A22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
avoid having empty distance in lessons list of each class and distribute quantities lessons each class has equally
</commit_message>
<xml_diff>
--- a/src/excel_resources/excel_data.xlsx
+++ b/src/excel_resources/excel_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18903091-5D99-4E82-B557-702971302EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2D3F16-CEA1-4EA5-AB6A-2727D7073BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1227,7 +1227,7 @@
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M7" s="13" t="str">
         <f t="shared" ref="M7:M31" si="0">F$116</f>
@@ -1258,7 +1258,7 @@
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M8" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1299,7 +1299,7 @@
         <v>85</v>
       </c>
       <c r="L9" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M9" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1329,7 +1329,7 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M10" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1360,7 +1360,7 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M11" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1390,7 +1390,7 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M12" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1421,7 +1421,7 @@
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M13" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1451,7 +1451,7 @@
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M14" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1482,7 +1482,7 @@
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
       <c r="L15" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M15" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1513,7 +1513,7 @@
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
       <c r="L16" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M16" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1544,7 +1544,7 @@
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
       <c r="L17" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M17" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1575,7 +1575,7 @@
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
       <c r="L18" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M18" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1606,7 +1606,7 @@
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
       <c r="L19" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M19" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1637,7 +1637,7 @@
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
       <c r="L20" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M20" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1667,7 +1667,7 @@
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
       <c r="L21" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M21" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1697,7 +1697,7 @@
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
       <c r="L22" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M22" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1727,7 +1727,7 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M23" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1765,7 +1765,7 @@
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
       <c r="L24" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M24" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1795,7 +1795,7 @@
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
       <c r="L25" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M25" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1825,7 +1825,7 @@
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
       <c r="L26" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M26" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1855,7 +1855,7 @@
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
       <c r="L27" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M27" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1885,7 +1885,7 @@
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
       <c r="L28" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M28" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1915,7 +1915,7 @@
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
       <c r="L29" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M29" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1945,7 +1945,7 @@
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
       <c r="L30" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M30" s="13" t="str">
         <f t="shared" si="0"/>
@@ -1975,7 +1975,7 @@
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
       <c r="L31" s="13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M31" s="13" t="str">
         <f t="shared" si="0"/>
@@ -2004,8 +2004,8 @@
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
-      <c r="L32" s="1" t="s">
-        <v>22</v>
+      <c r="L32" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M32" s="1" t="s">
         <v>36</v>
@@ -2033,8 +2033,8 @@
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
-      <c r="L33" s="1" t="s">
-        <v>22</v>
+      <c r="L33" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M33" s="1" t="s">
         <v>36</v>
@@ -2062,8 +2062,8 @@
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
-      <c r="L34" s="1" t="s">
-        <v>22</v>
+      <c r="L34" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M34" s="1" t="s">
         <v>36</v>
@@ -2091,8 +2091,8 @@
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
-      <c r="L35" s="1" t="s">
-        <v>22</v>
+      <c r="L35" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M35" s="1" t="s">
         <v>36</v>
@@ -2120,8 +2120,8 @@
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
       <c r="K36" s="1"/>
-      <c r="L36" s="1" t="s">
-        <v>22</v>
+      <c r="L36" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M36" s="1" t="s">
         <v>36</v>
@@ -2149,8 +2149,8 @@
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
-      <c r="L37" s="1" t="s">
-        <v>22</v>
+      <c r="L37" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M37" s="1" t="s">
         <v>36</v>
@@ -2178,8 +2178,8 @@
       <c r="I38" s="1"/>
       <c r="J38" s="1"/>
       <c r="K38" s="1"/>
-      <c r="L38" s="1" t="s">
-        <v>22</v>
+      <c r="L38" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M38" s="1" t="s">
         <v>36</v>
@@ -2207,8 +2207,8 @@
       <c r="I39" s="1"/>
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
-      <c r="L39" s="1" t="s">
-        <v>22</v>
+      <c r="L39" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M39" s="1" t="s">
         <v>36</v>
@@ -2236,8 +2236,8 @@
       <c r="I40" s="1"/>
       <c r="J40" s="1"/>
       <c r="K40" s="1"/>
-      <c r="L40" s="1" t="s">
-        <v>22</v>
+      <c r="L40" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M40" s="1" t="s">
         <v>36</v>
@@ -2265,8 +2265,8 @@
       <c r="I41" s="1"/>
       <c r="J41" s="1"/>
       <c r="K41" s="1"/>
-      <c r="L41" s="1" t="s">
-        <v>22</v>
+      <c r="L41" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M41" s="1" t="s">
         <v>36</v>
@@ -2294,8 +2294,8 @@
       <c r="I42" s="1"/>
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
-      <c r="L42" s="1" t="s">
-        <v>22</v>
+      <c r="L42" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M42" s="1" t="s">
         <v>36</v>
@@ -2323,8 +2323,8 @@
       <c r="I43" s="1"/>
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
-      <c r="L43" s="1" t="s">
-        <v>22</v>
+      <c r="L43" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M43" s="1" t="s">
         <v>36</v>
@@ -2352,8 +2352,8 @@
       <c r="I44" s="1"/>
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
-      <c r="L44" s="1" t="s">
-        <v>22</v>
+      <c r="L44" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M44" s="1" t="s">
         <v>36</v>
@@ -2381,8 +2381,8 @@
       <c r="I45" s="1"/>
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
-      <c r="L45" s="1" t="s">
-        <v>22</v>
+      <c r="L45" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M45" s="1" t="s">
         <v>36</v>
@@ -2410,8 +2410,8 @@
       <c r="I46" s="1"/>
       <c r="J46" s="1"/>
       <c r="K46" s="1"/>
-      <c r="L46" s="1" t="s">
-        <v>22</v>
+      <c r="L46" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M46" s="1" t="s">
         <v>36</v>
@@ -2439,8 +2439,8 @@
       <c r="I47" s="1"/>
       <c r="J47" s="1"/>
       <c r="K47" s="1"/>
-      <c r="L47" s="1" t="s">
-        <v>22</v>
+      <c r="L47" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M47" s="1" t="s">
         <v>36</v>
@@ -2468,8 +2468,8 @@
       <c r="I48" s="1"/>
       <c r="J48" s="1"/>
       <c r="K48" s="1"/>
-      <c r="L48" s="1" t="s">
-        <v>22</v>
+      <c r="L48" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M48" s="1" t="s">
         <v>36</v>
@@ -2497,8 +2497,8 @@
       <c r="I49" s="1"/>
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>
-      <c r="L49" s="1" t="s">
-        <v>22</v>
+      <c r="L49" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M49" s="1" t="s">
         <v>36</v>
@@ -2526,8 +2526,8 @@
       <c r="I50" s="1"/>
       <c r="J50" s="1"/>
       <c r="K50" s="1"/>
-      <c r="L50" s="1" t="s">
-        <v>22</v>
+      <c r="L50" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M50" s="1" t="s">
         <v>36</v>
@@ -2555,8 +2555,8 @@
       <c r="I51" s="1"/>
       <c r="J51" s="1"/>
       <c r="K51" s="1"/>
-      <c r="L51" s="1" t="s">
-        <v>22</v>
+      <c r="L51" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M51" s="1" t="s">
         <v>36</v>
@@ -2584,8 +2584,8 @@
       <c r="I52" s="1"/>
       <c r="J52" s="1"/>
       <c r="K52" s="1"/>
-      <c r="L52" s="1" t="s">
-        <v>22</v>
+      <c r="L52" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M52" s="1" t="s">
         <v>36</v>
@@ -2613,8 +2613,8 @@
       <c r="I53" s="1"/>
       <c r="J53" s="1"/>
       <c r="K53" s="1"/>
-      <c r="L53" s="1" t="s">
-        <v>22</v>
+      <c r="L53" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M53" s="1" t="s">
         <v>36</v>
@@ -2642,8 +2642,8 @@
       <c r="I54" s="1"/>
       <c r="J54" s="1"/>
       <c r="K54" s="1"/>
-      <c r="L54" s="1" t="s">
-        <v>22</v>
+      <c r="L54" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M54" s="1" t="s">
         <v>36</v>
@@ -2671,8 +2671,8 @@
       <c r="I55" s="1"/>
       <c r="J55" s="1"/>
       <c r="K55" s="1"/>
-      <c r="L55" s="1" t="s">
-        <v>22</v>
+      <c r="L55" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M55" s="1" t="s">
         <v>36</v>
@@ -2700,8 +2700,8 @@
       <c r="I56" s="1"/>
       <c r="J56" s="1"/>
       <c r="K56" s="1"/>
-      <c r="L56" s="1" t="s">
-        <v>22</v>
+      <c r="L56" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M56" s="1" t="s">
         <v>36</v>
@@ -2729,8 +2729,8 @@
       <c r="I57" s="1"/>
       <c r="J57" s="1"/>
       <c r="K57" s="1"/>
-      <c r="L57" s="1" t="s">
-        <v>22</v>
+      <c r="L57" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M57" s="1" t="s">
         <v>36</v>
@@ -2758,8 +2758,8 @@
       <c r="I58" s="1"/>
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
-      <c r="L58" s="1" t="s">
-        <v>22</v>
+      <c r="L58" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M58" s="1" t="s">
         <v>36</v>
@@ -2787,8 +2787,8 @@
       <c r="I59" s="1"/>
       <c r="J59" s="1"/>
       <c r="K59" s="1"/>
-      <c r="L59" s="1" t="s">
-        <v>22</v>
+      <c r="L59" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M59" s="1" t="s">
         <v>36</v>
@@ -2816,8 +2816,8 @@
       <c r="I60" s="1"/>
       <c r="J60" s="1"/>
       <c r="K60" s="1"/>
-      <c r="L60" s="1" t="s">
-        <v>22</v>
+      <c r="L60" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M60" s="1" t="s">
         <v>36</v>
@@ -2845,8 +2845,8 @@
       <c r="I61" s="1"/>
       <c r="J61" s="1"/>
       <c r="K61" s="1"/>
-      <c r="L61" s="1" t="s">
-        <v>22</v>
+      <c r="L61" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M61" s="1" t="s">
         <v>36</v>
@@ -2874,8 +2874,8 @@
       <c r="I62" s="1"/>
       <c r="J62" s="1"/>
       <c r="K62" s="1"/>
-      <c r="L62" s="1" t="s">
-        <v>24</v>
+      <c r="L62" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M62" s="1" t="s">
         <v>35</v>
@@ -2892,7 +2892,7 @@
         <v>61</v>
       </c>
       <c r="D63" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E63" s="1">
         <v>70</v>
@@ -2903,8 +2903,8 @@
       <c r="I63" s="1"/>
       <c r="J63" s="1"/>
       <c r="K63" s="1"/>
-      <c r="L63" s="1" t="s">
-        <v>24</v>
+      <c r="L63" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M63" s="1" t="s">
         <v>35</v>
@@ -2921,7 +2921,7 @@
         <v>61</v>
       </c>
       <c r="D64" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E64" s="1">
         <v>70</v>
@@ -2932,8 +2932,8 @@
       <c r="I64" s="1"/>
       <c r="J64" s="1"/>
       <c r="K64" s="1"/>
-      <c r="L64" s="1" t="s">
-        <v>24</v>
+      <c r="L64" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M64" s="1" t="s">
         <v>35</v>
@@ -2950,7 +2950,7 @@
         <v>61</v>
       </c>
       <c r="D65" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E65" s="1">
         <v>50</v>
@@ -2961,8 +2961,8 @@
       <c r="I65" s="1"/>
       <c r="J65" s="1"/>
       <c r="K65" s="1"/>
-      <c r="L65" s="1" t="s">
-        <v>24</v>
+      <c r="L65" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="M65" s="1" t="s">
         <v>35</v>
@@ -3637,7 +3637,7 @@
         <v>21</v>
       </c>
       <c r="D123" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E123" s="2" t="b">
         <f t="shared" si="2"/>
@@ -3659,7 +3659,7 @@
         <v>21</v>
       </c>
       <c r="D124" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E124" s="2" t="b">
         <f t="shared" si="2"/>
@@ -3703,7 +3703,7 @@
         <v>21</v>
       </c>
       <c r="D126" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E126" s="2" t="b">
         <f t="shared" si="2"/>
@@ -3725,7 +3725,7 @@
         <v>21</v>
       </c>
       <c r="D127" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E127" s="2" t="b">
         <f t="shared" si="2"/>
@@ -3747,7 +3747,7 @@
         <v>21</v>
       </c>
       <c r="D128" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E128" s="2" t="b">
         <f t="shared" si="2"/>
@@ -3769,7 +3769,7 @@
         <v>21</v>
       </c>
       <c r="D129" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E129" s="2" t="b">
         <f t="shared" si="2"/>
@@ -3837,7 +3837,7 @@
         <v>21</v>
       </c>
       <c r="D132" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E132" s="2" t="b">
         <v>0</v>
@@ -4145,10 +4145,10 @@
         <v>166</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>155</v>
+        <v>179</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="V6" s="1" t="s">
         <v>169</v>
@@ -4160,7 +4160,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>152</v>
@@ -4172,10 +4172,10 @@
         <v>154</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>157</v>
@@ -4187,37 +4187,37 @@
         <v>160</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>163</v>
+        <v>72</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="O7" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q7" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="P7" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>165</v>
-      </c>
       <c r="R7" s="1" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="S7" s="1" t="s">
         <v>166</v>
       </c>
       <c r="T7" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="V7" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
@@ -4226,64 +4226,64 @@
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>175</v>
+        <v>72</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>151</v>
+        <v>179</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>156</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>172</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>159</v>
+        <v>72</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>161</v>
+        <v>72</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>179</v>
+        <v>154</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>164</v>
+        <v>72</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q8" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="R8" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="R8" s="1" t="s">
-        <v>177</v>
-      </c>
       <c r="S8" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="T8" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="T8" s="1" t="s">
+      <c r="U8" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="V8" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
@@ -4292,43 +4292,43 @@
         <v>4</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>179</v>
+        <v>72</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>170</v>
+        <v>72</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>181</v>
+        <v>72</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>153</v>
+        <v>72</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>169</v>
+        <v>72</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>178</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>173</v>
+        <v>72</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>154</v>
+        <v>72</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>151</v>
+        <v>72</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>72</v>
@@ -4337,19 +4337,19 @@
         <v>155</v>
       </c>
       <c r="R9" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="S9" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="S9" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="T9" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>159</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
@@ -4358,10 +4358,10 @@
         <v>5</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>174</v>
+        <v>72</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>175</v>
+        <v>72</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>72</v>
@@ -4370,49 +4370,49 @@
         <v>72</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>153</v>
+        <v>72</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>196</v>
+        <v>72</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>176</v>
+        <v>72</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>173</v>
+        <v>72</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>154</v>
+        <v>72</v>
       </c>
       <c r="N10" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>159</v>
+        <v>72</v>
       </c>
       <c r="P10" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q10" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="S10" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T10" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="R10" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="S10" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="T10" s="1" t="s">
-        <v>179</v>
-      </c>
       <c r="U10" s="1" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="V10" s="1" t="s">
         <v>72</v>
@@ -4426,43 +4426,43 @@
         <v>6</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="E11" s="1" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>72</v>
+        <v>184</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>72</v>
+        <v>189</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>72</v>
+        <v>190</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>185</v>
       </c>
       <c r="K11" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O11" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="N11" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="O11" s="1" t="s">
-        <v>197</v>
       </c>
       <c r="P11" s="1" t="s">
         <v>72</v>
@@ -4492,19 +4492,19 @@
         <v>7</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="E12" s="1" t="s">
-        <v>188</v>
+        <v>72</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>72</v>
+        <v>189</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>72</v>
+        <v>190</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>72</v>
@@ -4513,13 +4513,13 @@
         <v>72</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>191</v>
+        <v>72</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>192</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>72</v>
+        <v>197</v>
       </c>
       <c r="M12" s="1" t="s">
         <v>72</v>
@@ -4567,7 +4567,7 @@
         <v>72</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>72</v>
+        <v>190</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>72</v>
@@ -4713,7 +4713,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>151</v>
+        <v>170</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>152</v>
@@ -4722,55 +4722,55 @@
         <v>153</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>175</v>
+        <v>154</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>157</v>
       </c>
       <c r="J18" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K18" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="L18" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="L18" s="1" t="s">
-        <v>169</v>
-      </c>
       <c r="M18" s="1" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="O18" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="P18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q18" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="P18" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q18" s="1" t="s">
-        <v>176</v>
-      </c>
       <c r="R18" s="1" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="S18" s="1" t="s">
         <v>166</v>
       </c>
       <c r="T18" s="1" t="s">
-        <v>72</v>
+        <v>176</v>
       </c>
       <c r="U18" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="V18" s="1" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
@@ -4779,64 +4779,64 @@
         <v>2</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="H19" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="I19" s="1" t="s">
-        <v>72</v>
+        <v>157</v>
       </c>
       <c r="J19" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K19" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="K19" s="1" t="s">
-        <v>164</v>
-      </c>
       <c r="L19" s="1" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="N19" s="1" t="s">
         <v>159</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="P19" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="S19" s="1" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="T19" s="1" t="s">
-        <v>72</v>
+        <v>162</v>
       </c>
       <c r="U19" s="1" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="V19" s="1" t="s">
-        <v>72</v>
+        <v>178</v>
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
@@ -4845,61 +4845,61 @@
         <v>3</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>175</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="J20" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K20" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="K20" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="L20" s="1" t="s">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>72</v>
+        <v>154</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>72</v>
+        <v>164</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q20" s="1" t="s">
-        <v>177</v>
+        <v>161</v>
       </c>
       <c r="R20" s="1" t="s">
-        <v>72</v>
+        <v>180</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="U20" s="1" t="s">
-        <v>72</v>
+        <v>157</v>
       </c>
       <c r="V20" s="1" t="s">
         <v>72</v>
@@ -4920,22 +4920,22 @@
         <v>72</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>72</v>
+        <v>152</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>72</v>
+        <v>168</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>72</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>72</v>
+        <v>178</v>
       </c>
       <c r="L21" s="1" t="s">
         <v>72</v>
@@ -4944,7 +4944,7 @@
         <v>72</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>72</v>
+        <v>154</v>
       </c>
       <c r="O21" s="1" t="s">
         <v>72</v>
@@ -4953,19 +4953,19 @@
         <v>72</v>
       </c>
       <c r="Q21" s="1" t="s">
-        <v>72</v>
+        <v>174</v>
       </c>
       <c r="R21" s="1" t="s">
-        <v>72</v>
+        <v>177</v>
       </c>
       <c r="S21" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="T21" s="1" t="s">
         <v>72</v>
       </c>
       <c r="U21" s="1" t="s">
-        <v>72</v>
+        <v>180</v>
       </c>
       <c r="V21" s="1" t="s">
         <v>72</v>
@@ -4995,13 +4995,13 @@
         <v>72</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>72</v>
+        <v>175</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>72</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="L22" s="1" t="s">
         <v>72</v>
@@ -5022,7 +5022,7 @@
         <v>72</v>
       </c>
       <c r="R22" s="1" t="s">
-        <v>72</v>
+        <v>177</v>
       </c>
       <c r="S22" s="1" t="s">
         <v>72</v>
@@ -5045,34 +5045,34 @@
         <v>6</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>72</v>
+        <v>193</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>72</v>
+        <v>188</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>72</v>
+        <v>183</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>72</v>
+        <v>187</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>72</v>
+        <v>184</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>72</v>
+        <v>189</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>72</v>
+        <v>191</v>
       </c>
       <c r="K23" s="1" t="s">
         <v>72</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>72</v>
+        <v>194</v>
       </c>
       <c r="M23" s="1" t="s">
         <v>186</v>
@@ -5117,7 +5117,7 @@
         <v>72</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>72</v>
+        <v>188</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>72</v>
@@ -5141,7 +5141,7 @@
         <v>72</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>72</v>
+        <v>197</v>
       </c>
       <c r="N24" s="1" t="s">
         <v>72</v>
@@ -5335,7 +5335,7 @@
         <v>170</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>179</v>
+        <v>151</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>152</v>
@@ -5347,49 +5347,49 @@
         <v>175</v>
       </c>
       <c r="H30" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="I30" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="I30" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="J30" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="K30" s="1" t="s">
         <v>154</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="M30" s="1" t="s">
         <v>159</v>
       </c>
       <c r="N30" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="O30" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="O30" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="P30" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q30" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="R30" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="R30" s="1" t="s">
+      <c r="S30" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="S30" s="1" t="s">
-        <v>155</v>
       </c>
       <c r="T30" s="1" t="s">
         <v>157</v>
       </c>
       <c r="U30" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="V30" s="1" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
@@ -5401,7 +5401,7 @@
         <v>174</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>152</v>
@@ -5410,52 +5410,52 @@
         <v>153</v>
       </c>
       <c r="G31" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="H31" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="H31" s="1" t="s">
-        <v>196</v>
-      </c>
       <c r="I31" s="1" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K31" s="1" t="s">
         <v>154</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>179</v>
+        <v>72</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>72</v>
+        <v>159</v>
       </c>
       <c r="P31" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q31" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="R31" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="R31" s="1" t="s">
-        <v>175</v>
-      </c>
       <c r="S31" s="1" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="T31" s="1" t="s">
         <v>157</v>
       </c>
       <c r="U31" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="V31" s="1" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
@@ -5464,64 +5464,64 @@
         <v>3</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>167</v>
+        <v>195</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>171</v>
+        <v>196</v>
       </c>
       <c r="G32" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I32" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="I32" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>161</v>
       </c>
       <c r="K32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="N32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="P32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q32" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="R32" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="S32" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="T32" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="L32" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="M32" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="N32" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="O32" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P32" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q32" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="R32" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="S32" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="T32" s="1" t="s">
+      <c r="U32" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="U32" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="V32" s="1" t="s">
-        <v>157</v>
+        <v>180</v>
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
@@ -5530,61 +5530,61 @@
         <v>4</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>177</v>
+        <v>72</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>173</v>
+        <v>195</v>
       </c>
       <c r="E33" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="G33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M33" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="G33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H33" s="1" t="s">
+      <c r="N33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q33" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="R33" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="S33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T33" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="U33" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="I33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="K33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L33" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="M33" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="N33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="O33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P33" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q33" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="R33" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="S33" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="T33" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="U33" s="1" t="s">
-        <v>179</v>
       </c>
       <c r="V33" s="1" t="s">
         <v>72</v>
@@ -5596,13 +5596,13 @@
         <v>5</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>167</v>
+        <v>72</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>72</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>174</v>
+        <v>72</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>72</v>
@@ -5611,19 +5611,19 @@
         <v>72</v>
       </c>
       <c r="H34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J34" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I34" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>178</v>
-      </c>
       <c r="K34" s="1" t="s">
         <v>72</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>169</v>
+        <v>72</v>
       </c>
       <c r="M34" s="1" t="s">
         <v>72</v>
@@ -5638,19 +5638,19 @@
         <v>72</v>
       </c>
       <c r="Q34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="U34" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="R34" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="S34" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="T34" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="U34" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="V34" s="1" t="s">
         <v>72</v>
@@ -5667,29 +5667,29 @@
         <v>72</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>193</v>
+        <v>72</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>72</v>
       </c>
       <c r="F35" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="K35" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G35" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="L35" s="1" t="s">
         <v>72</v>
       </c>
@@ -5697,10 +5697,10 @@
         <v>72</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>72</v>
+        <v>186</v>
       </c>
       <c r="O35" s="1" t="s">
-        <v>72</v>
+        <v>197</v>
       </c>
       <c r="P35" s="1" t="s">
         <v>72</v>
@@ -5733,7 +5733,7 @@
         <v>72</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>188</v>
+        <v>72</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>72</v>
@@ -5763,7 +5763,7 @@
         <v>72</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>72</v>
+        <v>197</v>
       </c>
       <c r="O36" s="1" t="s">
         <v>72</v>
@@ -5799,7 +5799,7 @@
         <v>72</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>182</v>
+        <v>72</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>72</v>
@@ -5951,19 +5951,19 @@
         <v>1</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>170</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>181</v>
+        <v>155</v>
       </c>
       <c r="H42" s="1" t="s">
         <v>171</v>
@@ -5972,19 +5972,19 @@
         <v>156</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>176</v>
+        <v>154</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>72</v>
+        <v>151</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>72</v>
+        <v>159</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="O42" s="1" t="s">
         <v>162</v>
@@ -5996,19 +5996,19 @@
         <v>158</v>
       </c>
       <c r="R42" s="1" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="S42" s="1" t="s">
         <v>165</v>
       </c>
       <c r="T42" s="1" t="s">
-        <v>178</v>
+        <v>157</v>
       </c>
       <c r="U42" s="1" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
       <c r="V42" s="1" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
@@ -6017,43 +6017,43 @@
         <v>2</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>195</v>
+        <v>179</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>174</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>72</v>
+        <v>152</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>72</v>
+        <v>181</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>196</v>
+        <v>155</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="K43" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="L43" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="M43" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="L43" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M43" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="N43" s="1" t="s">
-        <v>72</v>
+        <v>173</v>
       </c>
       <c r="O43" s="1" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="P43" s="1" t="s">
         <v>72</v>
@@ -6062,19 +6062,19 @@
         <v>158</v>
       </c>
       <c r="R43" s="1" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="S43" s="1" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="T43" s="1" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="U43" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="V43" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="V43" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
@@ -6083,19 +6083,19 @@
         <v>3</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>72</v>
+        <v>173</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>72</v>
+        <v>175</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>72</v>
+        <v>168</v>
       </c>
       <c r="H44" s="1" t="s">
         <v>72</v>
@@ -6104,16 +6104,16 @@
         <v>72</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>72</v>
+        <v>161</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>72</v>
+        <v>154</v>
       </c>
       <c r="N44" s="1" t="s">
         <v>72</v>
@@ -6125,22 +6125,22 @@
         <v>72</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="R44" s="1" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="S44" s="1" t="s">
-        <v>72</v>
+        <v>164</v>
       </c>
       <c r="T44" s="1" t="s">
-        <v>72</v>
+        <v>165</v>
       </c>
       <c r="U44" s="1" t="s">
-        <v>72</v>
+        <v>159</v>
       </c>
       <c r="V44" s="1" t="s">
-        <v>72</v>
+        <v>157</v>
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
@@ -6155,13 +6155,13 @@
         <v>72</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>72</v>
+        <v>181</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>72</v>
+        <v>168</v>
       </c>
       <c r="H45" s="1" t="s">
         <v>72</v>
@@ -6170,7 +6170,7 @@
         <v>72</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>72</v>
+        <v>176</v>
       </c>
       <c r="K45" s="1" t="s">
         <v>72</v>
@@ -6179,7 +6179,7 @@
         <v>72</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>72</v>
+        <v>169</v>
       </c>
       <c r="N45" s="1" t="s">
         <v>72</v>
@@ -6191,16 +6191,16 @@
         <v>72</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="R45" s="1" t="s">
-        <v>72</v>
+        <v>174</v>
       </c>
       <c r="S45" s="1" t="s">
-        <v>72</v>
+        <v>164</v>
       </c>
       <c r="T45" s="1" t="s">
-        <v>72</v>
+        <v>180</v>
       </c>
       <c r="U45" s="1" t="s">
         <v>72</v>
@@ -6236,7 +6236,7 @@
         <v>72</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="K46" s="1" t="s">
         <v>72</v>
@@ -6260,13 +6260,13 @@
         <v>72</v>
       </c>
       <c r="R46" s="1" t="s">
-        <v>72</v>
+        <v>180</v>
       </c>
       <c r="S46" s="1" t="s">
         <v>72</v>
       </c>
       <c r="T46" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="U46" s="1" t="s">
         <v>72</v>
@@ -6289,7 +6289,7 @@
         <v>72</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>193</v>
+        <v>72</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>72</v>
@@ -6316,10 +6316,10 @@
         <v>72</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>72</v>
+        <v>194</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>72</v>
+        <v>186</v>
       </c>
       <c r="P47" s="1" t="s">
         <v>72</v>
@@ -6385,7 +6385,7 @@
         <v>72</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>72</v>
+        <v>198</v>
       </c>
       <c r="P48" s="1" t="s">
         <v>72</v>
@@ -6570,64 +6570,64 @@
         <v>1</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D54" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="J54" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="L54" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M54" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N54" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="E54" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="H54" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="I54" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="J54" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="K54" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="L54" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="M54" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="N54" s="1" t="s">
+      <c r="O54" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="O54" s="1" t="s">
+      <c r="P54" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q54" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="P54" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q54" s="1" t="s">
+      <c r="R54" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="R54" s="1" t="s">
-        <v>164</v>
-      </c>
       <c r="S54" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="T54" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="T54" s="1" t="s">
+      <c r="U54" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="U54" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="V54" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
@@ -6636,64 +6636,64 @@
         <v>2</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>72</v>
+        <v>174</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>151</v>
+        <v>175</v>
       </c>
       <c r="F55" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="H55" s="1" t="s">
         <v>196</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="H55" s="1" t="s">
-        <v>155</v>
       </c>
       <c r="I55" s="1" t="s">
         <v>166</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="L55" s="1" t="s">
         <v>154</v>
       </c>
       <c r="M55" s="1" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="N55" s="1" t="s">
         <v>179</v>
       </c>
       <c r="O55" s="1" t="s">
-        <v>160</v>
+        <v>72</v>
       </c>
       <c r="P55" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q55" s="1" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="R55" s="1" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="S55" s="1" t="s">
         <v>161</v>
       </c>
       <c r="T55" s="1" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="U55" s="1" t="s">
         <v>165</v>
       </c>
       <c r="V55" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
@@ -6702,40 +6702,40 @@
         <v>3</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>173</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="F56" s="1" t="s">
-        <v>181</v>
-      </c>
       <c r="G56" s="1" t="s">
-        <v>152</v>
+        <v>196</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>72</v>
+        <v>164</v>
       </c>
       <c r="K56" s="1" t="s">
-        <v>178</v>
+        <v>159</v>
       </c>
       <c r="L56" s="1" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="M56" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="N56" s="1" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="O56" s="1" t="s">
         <v>72</v>
@@ -6744,19 +6744,19 @@
         <v>72</v>
       </c>
       <c r="Q56" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="R56" s="1" t="s">
         <v>161</v>
       </c>
       <c r="S56" s="1" t="s">
-        <v>164</v>
+        <v>72</v>
       </c>
       <c r="T56" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="U56" s="1" t="s">
-        <v>176</v>
+        <v>72</v>
       </c>
       <c r="V56" s="1" t="s">
         <v>177</v>
@@ -6768,64 +6768,64 @@
         <v>4</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>72</v>
+        <v>195</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>174</v>
+        <v>72</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>181</v>
+        <v>72</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>196</v>
+        <v>72</v>
       </c>
       <c r="H57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J57" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="K57" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="L57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="O57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="P57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q57" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="R57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T57" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="I57" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="K57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L57" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="M57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="N57" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="O57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="P57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="R57" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="S57" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="T57" s="1" t="s">
-        <v>180</v>
-      </c>
       <c r="U57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="V57" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="V57" s="1" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
@@ -6846,13 +6846,13 @@
         <v>72</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>152</v>
+        <v>72</v>
       </c>
       <c r="H58" s="1" t="s">
         <v>72</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="J58" s="1" t="s">
         <v>72</v>
@@ -6867,7 +6867,7 @@
         <v>72</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>154</v>
+        <v>72</v>
       </c>
       <c r="O58" s="1" t="s">
         <v>72</v>
@@ -6879,19 +6879,19 @@
         <v>72</v>
       </c>
       <c r="R58" s="1" t="s">
-        <v>155</v>
+        <v>72</v>
       </c>
       <c r="S58" s="1" t="s">
         <v>72</v>
       </c>
       <c r="T58" s="1" t="s">
-        <v>176</v>
+        <v>72</v>
       </c>
       <c r="U58" s="1" t="s">
-        <v>166</v>
+        <v>72</v>
       </c>
       <c r="V58" s="1" t="s">
-        <v>167</v>
+        <v>72</v>
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
@@ -6902,7 +6902,7 @@
         <v>6</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>188</v>
+        <v>72</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>72</v>
@@ -6911,34 +6911,34 @@
         <v>72</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>184</v>
+        <v>72</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>189</v>
+        <v>72</v>
       </c>
       <c r="H59" s="1" t="s">
         <v>72</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>200</v>
+        <v>72</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>199</v>
+        <v>72</v>
       </c>
       <c r="K59" s="1" t="s">
         <v>72</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>186</v>
+        <v>72</v>
       </c>
       <c r="M59" s="1" t="s">
         <v>187</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>194</v>
+        <v>72</v>
       </c>
       <c r="O59" s="1" t="s">
-        <v>198</v>
+        <v>72</v>
       </c>
       <c r="P59" s="1" t="s">
         <v>72</v>
@@ -6977,10 +6977,10 @@
         <v>72</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>189</v>
+        <v>72</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>190</v>
+        <v>72</v>
       </c>
       <c r="H60" s="1" t="s">
         <v>72</v>
@@ -6998,7 +6998,7 @@
         <v>72</v>
       </c>
       <c r="M60" s="1" t="s">
-        <v>197</v>
+        <v>72</v>
       </c>
       <c r="N60" s="1" t="s">
         <v>72</v>
@@ -7043,7 +7043,7 @@
         <v>72</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>190</v>
+        <v>72</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>72</v>
@@ -7064,7 +7064,7 @@
         <v>72</v>
       </c>
       <c r="M61" s="1" t="s">
-        <v>194</v>
+        <v>72</v>
       </c>
       <c r="N61" s="1" t="s">
         <v>72</v>
@@ -7189,13 +7189,13 @@
         <v>1</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>152</v>
@@ -7204,25 +7204,25 @@
         <v>153</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>196</v>
+        <v>155</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="J66" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="K66" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="K66" s="1" t="s">
-        <v>160</v>
       </c>
       <c r="L66" s="1" t="s">
         <v>154</v>
       </c>
       <c r="M66" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N66" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="N66" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="O66" s="1" t="s">
         <v>169</v>
@@ -7231,7 +7231,7 @@
         <v>72</v>
       </c>
       <c r="Q66" s="1" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="R66" s="1" t="s">
         <v>158</v>
@@ -7240,13 +7240,13 @@
         <v>162</v>
       </c>
       <c r="T66" s="1" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="U66" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="V66" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
@@ -7258,10 +7258,10 @@
         <v>173</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>195</v>
+        <v>174</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>152</v>
@@ -7270,49 +7270,49 @@
         <v>153</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>168</v>
+        <v>196</v>
       </c>
       <c r="J67" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="K67" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>169</v>
       </c>
       <c r="L67" s="1" t="s">
         <v>154</v>
       </c>
       <c r="M67" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N67" s="1" t="s">
         <v>171</v>
       </c>
       <c r="O67" s="1" t="s">
-        <v>151</v>
+        <v>72</v>
       </c>
       <c r="P67" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q67" s="1" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="R67" s="1" t="s">
         <v>158</v>
       </c>
       <c r="S67" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T67" s="1" t="s">
         <v>166</v>
       </c>
       <c r="U67" s="1" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="V67" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
@@ -7321,16 +7321,16 @@
         <v>3</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>72</v>
+        <v>173</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>195</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>151</v>
+        <v>175</v>
       </c>
       <c r="G68" s="1" t="s">
         <v>196</v>
@@ -7339,46 +7339,46 @@
         <v>72</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="K68" s="1" t="s">
-        <v>72</v>
+        <v>159</v>
       </c>
       <c r="L68" s="1" t="s">
-        <v>72</v>
+        <v>161</v>
       </c>
       <c r="M68" s="1" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="O68" s="1" t="s">
-        <v>160</v>
+        <v>72</v>
       </c>
       <c r="P68" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q68" s="1" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="R68" s="1" t="s">
         <v>155</v>
       </c>
       <c r="S68" s="1" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="T68" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="U68" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="V68" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="U68" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="V68" s="1" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
@@ -7390,22 +7390,22 @@
         <v>72</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>72</v>
+        <v>195</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>195</v>
+        <v>72</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="H69" s="1" t="s">
         <v>72</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>175</v>
+        <v>72</v>
       </c>
       <c r="J69" s="1" t="s">
         <v>72</v>
@@ -7417,31 +7417,31 @@
         <v>72</v>
       </c>
       <c r="M69" s="1" t="s">
-        <v>151</v>
+        <v>72</v>
       </c>
       <c r="N69" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O69" s="1" t="s">
-        <v>160</v>
+        <v>72</v>
       </c>
       <c r="P69" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q69" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R69" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="S69" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="R69" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="S69" s="1" t="s">
-        <v>164</v>
-      </c>
       <c r="T69" s="1" t="s">
-        <v>176</v>
+        <v>72</v>
       </c>
       <c r="U69" s="1" t="s">
-        <v>157</v>
+        <v>72</v>
       </c>
       <c r="V69" s="1" t="s">
         <v>167</v>
@@ -7459,10 +7459,10 @@
         <v>72</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>195</v>
+        <v>72</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>175</v>
+        <v>72</v>
       </c>
       <c r="G70" s="1" t="s">
         <v>72</v>
@@ -7471,7 +7471,7 @@
         <v>72</v>
       </c>
       <c r="I70" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="J70" s="1" t="s">
         <v>72</v>
@@ -7483,34 +7483,34 @@
         <v>72</v>
       </c>
       <c r="M70" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="N70" s="1" t="s">
         <v>72</v>
       </c>
       <c r="O70" s="1" t="s">
-        <v>159</v>
+        <v>72</v>
       </c>
       <c r="P70" s="1" t="s">
         <v>72</v>
       </c>
       <c r="Q70" s="1" t="s">
-        <v>177</v>
+        <v>72</v>
       </c>
       <c r="R70" s="1" t="s">
         <v>72</v>
       </c>
       <c r="S70" s="1" t="s">
-        <v>179</v>
+        <v>72</v>
       </c>
       <c r="T70" s="1" t="s">
-        <v>155</v>
+        <v>72</v>
       </c>
       <c r="U70" s="1" t="s">
-        <v>176</v>
+        <v>72</v>
       </c>
       <c r="V70" s="1" t="s">
-        <v>180</v>
+        <v>72</v>
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
@@ -7536,7 +7536,7 @@
         <v>72</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>184</v>
+        <v>72</v>
       </c>
       <c r="I71" s="1" t="s">
         <v>72</v>
@@ -7545,10 +7545,10 @@
         <v>72</v>
       </c>
       <c r="K71" s="1" t="s">
-        <v>191</v>
+        <v>72</v>
       </c>
       <c r="L71" s="1" t="s">
-        <v>197</v>
+        <v>72</v>
       </c>
       <c r="M71" s="1" t="s">
         <v>72</v>
@@ -7557,7 +7557,7 @@
         <v>187</v>
       </c>
       <c r="O71" s="1" t="s">
-        <v>186</v>
+        <v>72</v>
       </c>
       <c r="P71" s="1" t="s">
         <v>72</v>
@@ -7602,7 +7602,7 @@
         <v>72</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>189</v>
+        <v>72</v>
       </c>
       <c r="I72" s="1" t="s">
         <v>72</v>
@@ -7614,16 +7614,16 @@
         <v>72</v>
       </c>
       <c r="L72" s="1" t="s">
-        <v>194</v>
+        <v>72</v>
       </c>
       <c r="M72" s="1" t="s">
         <v>72</v>
       </c>
       <c r="N72" s="1" t="s">
-        <v>186</v>
+        <v>72</v>
       </c>
       <c r="O72" s="1" t="s">
-        <v>187</v>
+        <v>72</v>
       </c>
       <c r="P72" s="1" t="s">
         <v>72</v>
@@ -7686,7 +7686,7 @@
         <v>72</v>
       </c>
       <c r="N73" s="1" t="s">
-        <v>197</v>
+        <v>72</v>
       </c>
       <c r="O73" s="1" t="s">
         <v>72</v>

</xml_diff>

<commit_message>
adding is overcome max quantities continues same lessons
</commit_message>
<xml_diff>
--- a/src/excel_resources/excel_data.xlsx
+++ b/src/excel_resources/excel_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java memory\java learning\java project\TeacherWorkingDistributionSchedule\src\excel_resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2D3F16-CEA1-4EA5-AB6A-2727D7073BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA466B43-30DE-46CC-AB2B-2C7627C03C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="input" sheetId="1" r:id="rId1"/>
@@ -832,15 +832,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -852,6 +843,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4000,28 +4000,28 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20"/>
-      <c r="O4" s="20"/>
-      <c r="P4" s="20"/>
-      <c r="Q4" s="20"/>
-      <c r="R4" s="20"/>
-      <c r="S4" s="20"/>
-      <c r="T4" s="20"/>
-      <c r="U4" s="20"/>
-      <c r="V4" s="21"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="24"/>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
+      <c r="V4" s="25"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
@@ -4087,7 +4087,7 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="3">
@@ -4155,7 +4155,7 @@
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A7" s="22"/>
+      <c r="A7" s="19"/>
       <c r="B7" s="3">
         <v>2</v>
       </c>
@@ -4221,7 +4221,7 @@
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A8" s="22"/>
+      <c r="A8" s="19"/>
       <c r="B8" s="3">
         <v>3</v>
       </c>
@@ -4274,10 +4274,10 @@
         <v>174</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="U8" s="1" t="s">
         <v>157</v>
@@ -4287,7 +4287,7 @@
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A9" s="22"/>
+      <c r="A9" s="19"/>
       <c r="B9" s="3">
         <v>4</v>
       </c>
@@ -4310,7 +4310,7 @@
         <v>72</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>72</v>
+        <v>196</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>72</v>
@@ -4346,14 +4346,14 @@
         <v>168</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>167</v>
+        <v>72</v>
       </c>
       <c r="V9" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A10" s="22"/>
+      <c r="A10" s="19"/>
       <c r="B10" s="3">
         <v>5</v>
       </c>
@@ -4382,7 +4382,7 @@
         <v>72</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="L10" s="1" t="s">
         <v>72</v>
@@ -4406,20 +4406,20 @@
         <v>177</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="T10" s="1" t="s">
         <v>180</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>155</v>
+        <v>72</v>
       </c>
       <c r="V10" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="3">
@@ -4487,7 +4487,7 @@
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="24"/>
+      <c r="A12" s="21"/>
       <c r="B12" s="4">
         <v>7</v>
       </c>
@@ -4553,7 +4553,7 @@
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A13" s="25"/>
+      <c r="A13" s="22"/>
       <c r="B13" s="4">
         <v>8</v>
       </c>
@@ -4619,28 +4619,28 @@
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
-      <c r="L16" s="20"/>
-      <c r="M16" s="20"/>
-      <c r="N16" s="20"/>
-      <c r="O16" s="20"/>
-      <c r="P16" s="20"/>
-      <c r="Q16" s="20"/>
-      <c r="R16" s="20"/>
-      <c r="S16" s="20"/>
-      <c r="T16" s="20"/>
-      <c r="U16" s="20"/>
-      <c r="V16" s="21"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
+      <c r="L16" s="24"/>
+      <c r="M16" s="24"/>
+      <c r="N16" s="24"/>
+      <c r="O16" s="24"/>
+      <c r="P16" s="24"/>
+      <c r="Q16" s="24"/>
+      <c r="R16" s="24"/>
+      <c r="S16" s="24"/>
+      <c r="T16" s="24"/>
+      <c r="U16" s="24"/>
+      <c r="V16" s="25"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -4706,7 +4706,7 @@
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="3">
@@ -4774,7 +4774,7 @@
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A19" s="22"/>
+      <c r="A19" s="19"/>
       <c r="B19" s="3">
         <v>2</v>
       </c>
@@ -4840,7 +4840,7 @@
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A20" s="22"/>
+      <c r="A20" s="19"/>
       <c r="B20" s="3">
         <v>3</v>
       </c>
@@ -4878,7 +4878,7 @@
         <v>154</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="O20" s="1" t="s">
         <v>164</v>
@@ -4890,7 +4890,7 @@
         <v>161</v>
       </c>
       <c r="R20" s="1" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="S20" s="1" t="s">
         <v>178</v>
@@ -4902,11 +4902,11 @@
         <v>157</v>
       </c>
       <c r="V20" s="1" t="s">
-        <v>72</v>
+        <v>180</v>
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A21" s="22"/>
+      <c r="A21" s="19"/>
       <c r="B21" s="3">
         <v>4</v>
       </c>
@@ -4920,7 +4920,7 @@
         <v>72</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>155</v>
+        <v>72</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>152</v>
@@ -4944,7 +4944,7 @@
         <v>72</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>154</v>
+        <v>173</v>
       </c>
       <c r="O21" s="1" t="s">
         <v>72</v>
@@ -4953,13 +4953,13 @@
         <v>72</v>
       </c>
       <c r="Q21" s="1" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="R21" s="1" t="s">
         <v>177</v>
       </c>
       <c r="S21" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="T21" s="1" t="s">
         <v>72</v>
@@ -4972,7 +4972,7 @@
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A22" s="22"/>
+      <c r="A22" s="19"/>
       <c r="B22" s="3">
         <v>5</v>
       </c>
@@ -4995,13 +4995,13 @@
         <v>72</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>175</v>
+        <v>72</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>72</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="L22" s="1" t="s">
         <v>72</v>
@@ -5038,7 +5038,7 @@
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A23" s="23" t="s">
+      <c r="A23" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="3">
@@ -5106,7 +5106,7 @@
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A24" s="24"/>
+      <c r="A24" s="21"/>
       <c r="B24" s="4">
         <v>7</v>
       </c>
@@ -5172,7 +5172,7 @@
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A25" s="25"/>
+      <c r="A25" s="22"/>
       <c r="B25" s="4">
         <v>8</v>
       </c>
@@ -5238,28 +5238,28 @@
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C28" s="19" t="s">
+      <c r="C28" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="20"/>
-      <c r="J28" s="20"/>
-      <c r="K28" s="20"/>
-      <c r="L28" s="20"/>
-      <c r="M28" s="20"/>
-      <c r="N28" s="20"/>
-      <c r="O28" s="20"/>
-      <c r="P28" s="20"/>
-      <c r="Q28" s="20"/>
-      <c r="R28" s="20"/>
-      <c r="S28" s="20"/>
-      <c r="T28" s="20"/>
-      <c r="U28" s="20"/>
-      <c r="V28" s="21"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="24"/>
+      <c r="K28" s="24"/>
+      <c r="L28" s="24"/>
+      <c r="M28" s="24"/>
+      <c r="N28" s="24"/>
+      <c r="O28" s="24"/>
+      <c r="P28" s="24"/>
+      <c r="Q28" s="24"/>
+      <c r="R28" s="24"/>
+      <c r="S28" s="24"/>
+      <c r="T28" s="24"/>
+      <c r="U28" s="24"/>
+      <c r="V28" s="25"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B29" s="1"/>
@@ -5325,7 +5325,7 @@
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="22" t="s">
+      <c r="A30" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="3">
@@ -5393,7 +5393,7 @@
       </c>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A31" s="22"/>
+      <c r="A31" s="19"/>
       <c r="B31" s="3">
         <v>2</v>
       </c>
@@ -5459,7 +5459,7 @@
       </c>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A32" s="22"/>
+      <c r="A32" s="19"/>
       <c r="B32" s="3">
         <v>3</v>
       </c>
@@ -5482,7 +5482,7 @@
         <v>72</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>161</v>
@@ -5521,11 +5521,11 @@
         <v>162</v>
       </c>
       <c r="V32" s="1" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="22"/>
+      <c r="A33" s="19"/>
       <c r="B33" s="3">
         <v>4</v>
       </c>
@@ -5548,7 +5548,7 @@
         <v>72</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>178</v>
@@ -5566,7 +5566,7 @@
         <v>72</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>72</v>
+        <v>154</v>
       </c>
       <c r="P33" s="1" t="s">
         <v>72</v>
@@ -5587,11 +5587,11 @@
         <v>155</v>
       </c>
       <c r="V33" s="1" t="s">
-        <v>72</v>
+        <v>168</v>
       </c>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" s="22"/>
+      <c r="A34" s="19"/>
       <c r="B34" s="3">
         <v>5</v>
       </c>
@@ -5614,7 +5614,7 @@
         <v>72</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>171</v>
@@ -5641,7 +5641,7 @@
         <v>72</v>
       </c>
       <c r="R34" s="1" t="s">
-        <v>72</v>
+        <v>180</v>
       </c>
       <c r="S34" s="1" t="s">
         <v>72</v>
@@ -5650,14 +5650,14 @@
         <v>72</v>
       </c>
       <c r="U34" s="1" t="s">
-        <v>180</v>
+        <v>72</v>
       </c>
       <c r="V34" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" s="23" t="s">
+      <c r="A35" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="3">
@@ -5725,7 +5725,7 @@
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="24"/>
+      <c r="A36" s="21"/>
       <c r="B36" s="4">
         <v>7</v>
       </c>
@@ -5791,7 +5791,7 @@
       </c>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="25"/>
+      <c r="A37" s="22"/>
       <c r="B37" s="4">
         <v>8</v>
       </c>
@@ -5857,28 +5857,28 @@
       </c>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C40" s="19" t="s">
+      <c r="C40" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="20"/>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20"/>
-      <c r="I40" s="20"/>
-      <c r="J40" s="20"/>
-      <c r="K40" s="20"/>
-      <c r="L40" s="20"/>
-      <c r="M40" s="20"/>
-      <c r="N40" s="20"/>
-      <c r="O40" s="20"/>
-      <c r="P40" s="20"/>
-      <c r="Q40" s="20"/>
-      <c r="R40" s="20"/>
-      <c r="S40" s="20"/>
-      <c r="T40" s="20"/>
-      <c r="U40" s="20"/>
-      <c r="V40" s="21"/>
+      <c r="D40" s="24"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="24"/>
+      <c r="G40" s="24"/>
+      <c r="H40" s="24"/>
+      <c r="I40" s="24"/>
+      <c r="J40" s="24"/>
+      <c r="K40" s="24"/>
+      <c r="L40" s="24"/>
+      <c r="M40" s="24"/>
+      <c r="N40" s="24"/>
+      <c r="O40" s="24"/>
+      <c r="P40" s="24"/>
+      <c r="Q40" s="24"/>
+      <c r="R40" s="24"/>
+      <c r="S40" s="24"/>
+      <c r="T40" s="24"/>
+      <c r="U40" s="24"/>
+      <c r="V40" s="25"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B41" s="1"/>
@@ -5944,7 +5944,7 @@
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="22" t="s">
+      <c r="A42" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B42" s="3">
@@ -6012,7 +6012,7 @@
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="22"/>
+      <c r="A43" s="19"/>
       <c r="B43" s="3">
         <v>2</v>
       </c>
@@ -6078,7 +6078,7 @@
       </c>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="22"/>
+      <c r="A44" s="19"/>
       <c r="B44" s="3">
         <v>3</v>
       </c>
@@ -6144,7 +6144,7 @@
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" s="22"/>
+      <c r="A45" s="19"/>
       <c r="B45" s="3">
         <v>4</v>
       </c>
@@ -6158,7 +6158,7 @@
         <v>181</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>171</v>
+        <v>155</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>168</v>
@@ -6173,7 +6173,7 @@
         <v>176</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="L45" s="1" t="s">
         <v>72</v>
@@ -6191,26 +6191,26 @@
         <v>72</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="R45" s="1" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="S45" s="1" t="s">
         <v>164</v>
       </c>
       <c r="T45" s="1" t="s">
-        <v>180</v>
+        <v>72</v>
       </c>
       <c r="U45" s="1" t="s">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="V45" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A46" s="22"/>
+      <c r="A46" s="19"/>
       <c r="B46" s="3">
         <v>5</v>
       </c>
@@ -6260,23 +6260,23 @@
         <v>72</v>
       </c>
       <c r="R46" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S46" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T46" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="U46" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="S46" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="T46" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="U46" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="V46" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="23" t="s">
+      <c r="A47" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B47" s="3">
@@ -6344,7 +6344,7 @@
       </c>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="24"/>
+      <c r="A48" s="21"/>
       <c r="B48" s="4">
         <v>7</v>
       </c>
@@ -6410,7 +6410,7 @@
       </c>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A49" s="25"/>
+      <c r="A49" s="22"/>
       <c r="B49" s="4">
         <v>8</v>
       </c>
@@ -6476,28 +6476,28 @@
       </c>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C52" s="19" t="s">
+      <c r="C52" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="20"/>
-      <c r="E52" s="20"/>
-      <c r="F52" s="20"/>
-      <c r="G52" s="20"/>
-      <c r="H52" s="20"/>
-      <c r="I52" s="20"/>
-      <c r="J52" s="20"/>
-      <c r="K52" s="20"/>
-      <c r="L52" s="20"/>
-      <c r="M52" s="20"/>
-      <c r="N52" s="20"/>
-      <c r="O52" s="20"/>
-      <c r="P52" s="20"/>
-      <c r="Q52" s="20"/>
-      <c r="R52" s="20"/>
-      <c r="S52" s="20"/>
-      <c r="T52" s="20"/>
-      <c r="U52" s="20"/>
-      <c r="V52" s="21"/>
+      <c r="D52" s="24"/>
+      <c r="E52" s="24"/>
+      <c r="F52" s="24"/>
+      <c r="G52" s="24"/>
+      <c r="H52" s="24"/>
+      <c r="I52" s="24"/>
+      <c r="J52" s="24"/>
+      <c r="K52" s="24"/>
+      <c r="L52" s="24"/>
+      <c r="M52" s="24"/>
+      <c r="N52" s="24"/>
+      <c r="O52" s="24"/>
+      <c r="P52" s="24"/>
+      <c r="Q52" s="24"/>
+      <c r="R52" s="24"/>
+      <c r="S52" s="24"/>
+      <c r="T52" s="24"/>
+      <c r="U52" s="24"/>
+      <c r="V52" s="25"/>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B53" s="1"/>
@@ -6563,7 +6563,7 @@
       </c>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A54" s="22" t="s">
+      <c r="A54" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="3">
@@ -6631,7 +6631,7 @@
       </c>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A55" s="22"/>
+      <c r="A55" s="19"/>
       <c r="B55" s="3">
         <v>2</v>
       </c>
@@ -6651,7 +6651,7 @@
         <v>153</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>196</v>
+        <v>155</v>
       </c>
       <c r="I55" s="1" t="s">
         <v>166</v>
@@ -6669,7 +6669,7 @@
         <v>160</v>
       </c>
       <c r="N55" s="1" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="O55" s="1" t="s">
         <v>72</v>
@@ -6684,10 +6684,10 @@
         <v>158</v>
       </c>
       <c r="S55" s="1" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="T55" s="1" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="U55" s="1" t="s">
         <v>165</v>
@@ -6697,7 +6697,7 @@
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A56" s="22"/>
+      <c r="A56" s="19"/>
       <c r="B56" s="3">
         <v>3</v>
       </c>
@@ -6763,7 +6763,7 @@
       </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" s="22"/>
+      <c r="A57" s="19"/>
       <c r="B57" s="3">
         <v>4</v>
       </c>
@@ -6771,13 +6771,13 @@
         <v>195</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>173</v>
+        <v>72</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>72</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>72</v>
+        <v>171</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>72</v>
@@ -6792,7 +6792,7 @@
         <v>178</v>
       </c>
       <c r="K57" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="L57" s="1" t="s">
         <v>72</v>
@@ -6819,7 +6819,7 @@
         <v>72</v>
       </c>
       <c r="T57" s="1" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="U57" s="1" t="s">
         <v>72</v>
@@ -6829,7 +6829,7 @@
       </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A58" s="22"/>
+      <c r="A58" s="19"/>
       <c r="B58" s="3">
         <v>5</v>
       </c>
@@ -6895,7 +6895,7 @@
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="23" t="s">
+      <c r="A59" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B59" s="3">
@@ -6963,7 +6963,7 @@
       </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="24"/>
+      <c r="A60" s="21"/>
       <c r="B60" s="4">
         <v>7</v>
       </c>
@@ -7029,7 +7029,7 @@
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="25"/>
+      <c r="A61" s="22"/>
       <c r="B61" s="4">
         <v>8</v>
       </c>
@@ -7095,28 +7095,28 @@
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="C64" s="19" t="s">
+      <c r="C64" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="D64" s="20"/>
-      <c r="E64" s="20"/>
-      <c r="F64" s="20"/>
-      <c r="G64" s="20"/>
-      <c r="H64" s="20"/>
-      <c r="I64" s="20"/>
-      <c r="J64" s="20"/>
-      <c r="K64" s="20"/>
-      <c r="L64" s="20"/>
-      <c r="M64" s="20"/>
-      <c r="N64" s="20"/>
-      <c r="O64" s="20"/>
-      <c r="P64" s="20"/>
-      <c r="Q64" s="20"/>
-      <c r="R64" s="20"/>
-      <c r="S64" s="20"/>
-      <c r="T64" s="20"/>
-      <c r="U64" s="20"/>
-      <c r="V64" s="21"/>
+      <c r="D64" s="24"/>
+      <c r="E64" s="24"/>
+      <c r="F64" s="24"/>
+      <c r="G64" s="24"/>
+      <c r="H64" s="24"/>
+      <c r="I64" s="24"/>
+      <c r="J64" s="24"/>
+      <c r="K64" s="24"/>
+      <c r="L64" s="24"/>
+      <c r="M64" s="24"/>
+      <c r="N64" s="24"/>
+      <c r="O64" s="24"/>
+      <c r="P64" s="24"/>
+      <c r="Q64" s="24"/>
+      <c r="R64" s="24"/>
+      <c r="S64" s="24"/>
+      <c r="T64" s="24"/>
+      <c r="U64" s="24"/>
+      <c r="V64" s="25"/>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B65" s="1"/>
@@ -7182,7 +7182,7 @@
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="22" t="s">
+      <c r="A66" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B66" s="3">
@@ -7250,7 +7250,7 @@
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="22"/>
+      <c r="A67" s="19"/>
       <c r="B67" s="3">
         <v>2</v>
       </c>
@@ -7270,10 +7270,10 @@
         <v>153</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>155</v>
+        <v>196</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>196</v>
+        <v>175</v>
       </c>
       <c r="J67" s="1" t="s">
         <v>169</v>
@@ -7303,7 +7303,7 @@
         <v>158</v>
       </c>
       <c r="S67" s="1" t="s">
-        <v>175</v>
+        <v>155</v>
       </c>
       <c r="T67" s="1" t="s">
         <v>166</v>
@@ -7316,7 +7316,7 @@
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" s="22"/>
+      <c r="A68" s="19"/>
       <c r="B68" s="3">
         <v>3</v>
       </c>
@@ -7339,7 +7339,7 @@
         <v>72</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
       <c r="J68" s="1" t="s">
         <v>164</v>
@@ -7382,7 +7382,7 @@
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="22"/>
+      <c r="A69" s="19"/>
       <c r="B69" s="3">
         <v>4</v>
       </c>
@@ -7390,7 +7390,7 @@
         <v>72</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>195</v>
+        <v>173</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>72</v>
@@ -7420,7 +7420,7 @@
         <v>72</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>72</v>
+        <v>179</v>
       </c>
       <c r="O69" s="1" t="s">
         <v>72</v>
@@ -7435,20 +7435,20 @@
         <v>161</v>
       </c>
       <c r="S69" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T69" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="U69" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="T69" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="U69" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="V69" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="22"/>
+      <c r="A70" s="19"/>
       <c r="B70" s="3">
         <v>5</v>
       </c>
@@ -7514,7 +7514,7 @@
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A71" s="23" t="s">
+      <c r="A71" s="20" t="s">
         <v>21</v>
       </c>
       <c r="B71" s="3">
@@ -7582,7 +7582,7 @@
       </c>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="24"/>
+      <c r="A72" s="21"/>
       <c r="B72" s="4">
         <v>7</v>
       </c>
@@ -7648,7 +7648,7 @@
       </c>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" s="25"/>
+      <c r="A73" s="22"/>
       <c r="B73" s="4">
         <v>8</v>
       </c>
@@ -7715,6 +7715,16 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C4:V4"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="C16:V16"/>
+    <mergeCell ref="A18:A22"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C28:V28"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="C64:V64"/>
     <mergeCell ref="A66:A70"/>
     <mergeCell ref="A71:A73"/>
     <mergeCell ref="C40:V40"/>
@@ -7723,16 +7733,6 @@
     <mergeCell ref="C52:V52"/>
     <mergeCell ref="A54:A58"/>
     <mergeCell ref="A59:A61"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="C28:V28"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="C64:V64"/>
-    <mergeCell ref="C4:V4"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="C16:V16"/>
-    <mergeCell ref="A18:A22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>